<commit_message>
Fix V3 core formulas and summary links for Down/Up engine
</commit_message>
<xml_diff>
--- a/MinusLock_Percent_Grid_Calculator/MinusLock_Percent_Grid_Calculator.xlsx
+++ b/MinusLock_Percent_Grid_Calculator/MinusLock_Percent_Grid_Calculator.xlsx
@@ -1898,27 +1898,30 @@
           <t>Strong Downtrend</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>35</v>
-      </c>
-      <c r="C4" t="n">
-        <v>9</v>
+      <c r="B4">
+        <f>25+AdaptiveEngine!B17/4</f>
+        <v/>
+      </c>
+      <c r="C4">
+        <f>INT(5+AdaptiveEngine!B17/20)</f>
+        <v/>
       </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>WARNING</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>850</v>
-      </c>
-      <c r="F4" t="n">
-        <v>420</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
+      <c r="E4">
+        <f>500+AdaptiveEngine!B17*6</f>
+        <v/>
+      </c>
+      <c r="F4">
+        <f>200+AdaptiveEngine!D17*8</f>
+        <v/>
+      </c>
+      <c r="G4">
+        <f>IF(B4&gt;60,"LOW","MEDIUM")</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -3056,7 +3059,7 @@
         <v/>
       </c>
       <c r="AA3">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G3/100,IF(Settings!$B$9,CEILING(MAX(0,V3+Settings!$B$2*G3/100-X3-Settings!$B$2*J3/100),Settings!$B$5),MAX(0,V3+Settings!$B$2*G3/100-X3-Settings!$B$2*J3/100))),IF(Settings!$B$9,MROUND(Z3,Settings!$B$5),Z3))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G3/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H3-I3+J3)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H3-I3+J3)/100))),IF(Settings!$B$9,MROUND(Z3,Settings!$B$5),Z3))</f>
         <v/>
       </c>
       <c r="AB3">
@@ -3173,7 +3176,7 @@
         <v/>
       </c>
       <c r="AA4">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G4/100,IF(Settings!$B$9,CEILING(MAX(0,V4+Settings!$B$2*G4/100-X4-Settings!$B$2*J4/100),Settings!$B$5),MAX(0,V4+Settings!$B$2*G4/100-X4-Settings!$B$2*J4/100))),IF(Settings!$B$9,MROUND(Z4,Settings!$B$5),Z4))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G4/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H4-I4+J4)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H4-I4+J4)/100))),IF(Settings!$B$9,MROUND(Z4,Settings!$B$5),Z4))</f>
         <v/>
       </c>
       <c r="AB4">
@@ -3290,7 +3293,7 @@
         <v/>
       </c>
       <c r="AA5">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G5/100,IF(Settings!$B$9,CEILING(MAX(0,V5+Settings!$B$2*G5/100-X5-Settings!$B$2*J5/100),Settings!$B$5),MAX(0,V5+Settings!$B$2*G5/100-X5-Settings!$B$2*J5/100))),IF(Settings!$B$9,MROUND(Z5,Settings!$B$5),Z5))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G5/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H5-I5+J5)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H5-I5+J5)/100))),IF(Settings!$B$9,MROUND(Z5,Settings!$B$5),Z5))</f>
         <v/>
       </c>
       <c r="AB5">
@@ -3407,7 +3410,7 @@
         <v/>
       </c>
       <c r="AA6">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G6/100,IF(Settings!$B$9,CEILING(MAX(0,V6+Settings!$B$2*G6/100-X6-Settings!$B$2*J6/100),Settings!$B$5),MAX(0,V6+Settings!$B$2*G6/100-X6-Settings!$B$2*J6/100))),IF(Settings!$B$9,MROUND(Z6,Settings!$B$5),Z6))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G6/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H6-I6+J6)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H6-I6+J6)/100))),IF(Settings!$B$9,MROUND(Z6,Settings!$B$5),Z6))</f>
         <v/>
       </c>
       <c r="AB6">
@@ -3524,7 +3527,7 @@
         <v/>
       </c>
       <c r="AA7">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G7/100,IF(Settings!$B$9,CEILING(MAX(0,V7+Settings!$B$2*G7/100-X7-Settings!$B$2*J7/100),Settings!$B$5),MAX(0,V7+Settings!$B$2*G7/100-X7-Settings!$B$2*J7/100))),IF(Settings!$B$9,MROUND(Z7,Settings!$B$5),Z7))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G7/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H7-I7+J7)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H7-I7+J7)/100))),IF(Settings!$B$9,MROUND(Z7,Settings!$B$5),Z7))</f>
         <v/>
       </c>
       <c r="AB7">
@@ -3641,7 +3644,7 @@
         <v/>
       </c>
       <c r="AA8">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G8/100,IF(Settings!$B$9,CEILING(MAX(0,V8+Settings!$B$2*G8/100-X8-Settings!$B$2*J8/100),Settings!$B$5),MAX(0,V8+Settings!$B$2*G8/100-X8-Settings!$B$2*J8/100))),IF(Settings!$B$9,MROUND(Z8,Settings!$B$5),Z8))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G8/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H8-I8+J8)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H8-I8+J8)/100))),IF(Settings!$B$9,MROUND(Z8,Settings!$B$5),Z8))</f>
         <v/>
       </c>
       <c r="AB8">
@@ -3758,7 +3761,7 @@
         <v/>
       </c>
       <c r="AA9">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G9/100,IF(Settings!$B$9,CEILING(MAX(0,V9+Settings!$B$2*G9/100-X9-Settings!$B$2*J9/100),Settings!$B$5),MAX(0,V9+Settings!$B$2*G9/100-X9-Settings!$B$2*J9/100))),IF(Settings!$B$9,MROUND(Z9,Settings!$B$5),Z9))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G9/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H9-I9+J9)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H9-I9+J9)/100))),IF(Settings!$B$9,MROUND(Z9,Settings!$B$5),Z9))</f>
         <v/>
       </c>
       <c r="AB9">
@@ -3875,7 +3878,7 @@
         <v/>
       </c>
       <c r="AA10">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G10/100,IF(Settings!$B$9,CEILING(MAX(0,V10+Settings!$B$2*G10/100-X10-Settings!$B$2*J10/100),Settings!$B$5),MAX(0,V10+Settings!$B$2*G10/100-X10-Settings!$B$2*J10/100))),IF(Settings!$B$9,MROUND(Z10,Settings!$B$5),Z10))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G10/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H10-I10+J10)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H10-I10+J10)/100))),IF(Settings!$B$9,MROUND(Z10,Settings!$B$5),Z10))</f>
         <v/>
       </c>
       <c r="AB10">
@@ -3992,7 +3995,7 @@
         <v/>
       </c>
       <c r="AA11">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G11/100,IF(Settings!$B$9,CEILING(MAX(0,V11+Settings!$B$2*G11/100-X11-Settings!$B$2*J11/100),Settings!$B$5),MAX(0,V11+Settings!$B$2*G11/100-X11-Settings!$B$2*J11/100))),IF(Settings!$B$9,MROUND(Z11,Settings!$B$5),Z11))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G11/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H11-I11+J11)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H11-I11+J11)/100))),IF(Settings!$B$9,MROUND(Z11,Settings!$B$5),Z11))</f>
         <v/>
       </c>
       <c r="AB11">
@@ -4109,7 +4112,7 @@
         <v/>
       </c>
       <c r="AA12">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G12/100,IF(Settings!$B$9,CEILING(MAX(0,V12+Settings!$B$2*G12/100-X12-Settings!$B$2*J12/100),Settings!$B$5),MAX(0,V12+Settings!$B$2*G12/100-X12-Settings!$B$2*J12/100))),IF(Settings!$B$9,MROUND(Z12,Settings!$B$5),Z12))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G12/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H12-I12+J12)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H12-I12+J12)/100))),IF(Settings!$B$9,MROUND(Z12,Settings!$B$5),Z12))</f>
         <v/>
       </c>
       <c r="AB12">
@@ -4226,7 +4229,7 @@
         <v/>
       </c>
       <c r="AA13">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G13/100,IF(Settings!$B$9,CEILING(MAX(0,V13+Settings!$B$2*G13/100-X13-Settings!$B$2*J13/100),Settings!$B$5),MAX(0,V13+Settings!$B$2*G13/100-X13-Settings!$B$2*J13/100))),IF(Settings!$B$9,MROUND(Z13,Settings!$B$5),Z13))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G13/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H13-I13+J13)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H13-I13+J13)/100))),IF(Settings!$B$9,MROUND(Z13,Settings!$B$5),Z13))</f>
         <v/>
       </c>
       <c r="AB13">
@@ -4343,7 +4346,7 @@
         <v/>
       </c>
       <c r="AA14">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G14/100,IF(Settings!$B$9,CEILING(MAX(0,V14+Settings!$B$2*G14/100-X14-Settings!$B$2*J14/100),Settings!$B$5),MAX(0,V14+Settings!$B$2*G14/100-X14-Settings!$B$2*J14/100))),IF(Settings!$B$9,MROUND(Z14,Settings!$B$5),Z14))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G14/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H14-I14+J14)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H14-I14+J14)/100))),IF(Settings!$B$9,MROUND(Z14,Settings!$B$5),Z14))</f>
         <v/>
       </c>
       <c r="AB14">
@@ -4460,7 +4463,7 @@
         <v/>
       </c>
       <c r="AA15">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G15/100,IF(Settings!$B$9,CEILING(MAX(0,V15+Settings!$B$2*G15/100-X15-Settings!$B$2*J15/100),Settings!$B$5),MAX(0,V15+Settings!$B$2*G15/100-X15-Settings!$B$2*J15/100))),IF(Settings!$B$9,MROUND(Z15,Settings!$B$5),Z15))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G15/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H15-I15+J15)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H15-I15+J15)/100))),IF(Settings!$B$9,MROUND(Z15,Settings!$B$5),Z15))</f>
         <v/>
       </c>
       <c r="AB15">
@@ -4577,7 +4580,7 @@
         <v/>
       </c>
       <c r="AA16">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G16/100,IF(Settings!$B$9,CEILING(MAX(0,V16+Settings!$B$2*G16/100-X16-Settings!$B$2*J16/100),Settings!$B$5),MAX(0,V16+Settings!$B$2*G16/100-X16-Settings!$B$2*J16/100))),IF(Settings!$B$9,MROUND(Z16,Settings!$B$5),Z16))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G16/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H16-I16+J16)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H16-I16+J16)/100))),IF(Settings!$B$9,MROUND(Z16,Settings!$B$5),Z16))</f>
         <v/>
       </c>
       <c r="AB16">
@@ -4694,7 +4697,7 @@
         <v/>
       </c>
       <c r="AA17">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G17/100,IF(Settings!$B$9,CEILING(MAX(0,V17+Settings!$B$2*G17/100-X17-Settings!$B$2*J17/100),Settings!$B$5),MAX(0,V17+Settings!$B$2*G17/100-X17-Settings!$B$2*J17/100))),IF(Settings!$B$9,MROUND(Z17,Settings!$B$5),Z17))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G17/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H17-I17+J17)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H17-I17+J17)/100))),IF(Settings!$B$9,MROUND(Z17,Settings!$B$5),Z17))</f>
         <v/>
       </c>
       <c r="AB17">
@@ -4811,7 +4814,7 @@
         <v/>
       </c>
       <c r="AA18">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G18/100,IF(Settings!$B$9,CEILING(MAX(0,V18+Settings!$B$2*G18/100-X18-Settings!$B$2*J18/100),Settings!$B$5),MAX(0,V18+Settings!$B$2*G18/100-X18-Settings!$B$2*J18/100))),IF(Settings!$B$9,MROUND(Z18,Settings!$B$5),Z18))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G18/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H18-I18+J18)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H18-I18+J18)/100))),IF(Settings!$B$9,MROUND(Z18,Settings!$B$5),Z18))</f>
         <v/>
       </c>
       <c r="AB18">
@@ -4928,7 +4931,7 @@
         <v/>
       </c>
       <c r="AA19">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G19/100,IF(Settings!$B$9,CEILING(MAX(0,V19+Settings!$B$2*G19/100-X19-Settings!$B$2*J19/100),Settings!$B$5),MAX(0,V19+Settings!$B$2*G19/100-X19-Settings!$B$2*J19/100))),IF(Settings!$B$9,MROUND(Z19,Settings!$B$5),Z19))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G19/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H19-I19+J19)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H19-I19+J19)/100))),IF(Settings!$B$9,MROUND(Z19,Settings!$B$5),Z19))</f>
         <v/>
       </c>
       <c r="AB19">
@@ -5045,7 +5048,7 @@
         <v/>
       </c>
       <c r="AA20">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G20/100,IF(Settings!$B$9,CEILING(MAX(0,V20+Settings!$B$2*G20/100-X20-Settings!$B$2*J20/100),Settings!$B$5),MAX(0,V20+Settings!$B$2*G20/100-X20-Settings!$B$2*J20/100))),IF(Settings!$B$9,MROUND(Z20,Settings!$B$5),Z20))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G20/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H20-I20+J20)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H20-I20+J20)/100))),IF(Settings!$B$9,MROUND(Z20,Settings!$B$5),Z20))</f>
         <v/>
       </c>
       <c r="AB20">
@@ -5162,7 +5165,7 @@
         <v/>
       </c>
       <c r="AA21">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G21/100,IF(Settings!$B$9,CEILING(MAX(0,V21+Settings!$B$2*G21/100-X21-Settings!$B$2*J21/100),Settings!$B$5),MAX(0,V21+Settings!$B$2*G21/100-X21-Settings!$B$2*J21/100))),IF(Settings!$B$9,MROUND(Z21,Settings!$B$5),Z21))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G21/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H21-I21+J21)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H21-I21+J21)/100))),IF(Settings!$B$9,MROUND(Z21,Settings!$B$5),Z21))</f>
         <v/>
       </c>
       <c r="AB21">
@@ -5279,7 +5282,7 @@
         <v/>
       </c>
       <c r="AA22">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G22/100,IF(Settings!$B$9,CEILING(MAX(0,V22+Settings!$B$2*G22/100-X22-Settings!$B$2*J22/100),Settings!$B$5),MAX(0,V22+Settings!$B$2*G22/100-X22-Settings!$B$2*J22/100))),IF(Settings!$B$9,MROUND(Z22,Settings!$B$5),Z22))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G22/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H22-I22+J22)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H22-I22+J22)/100))),IF(Settings!$B$9,MROUND(Z22,Settings!$B$5),Z22))</f>
         <v/>
       </c>
       <c r="AB22">
@@ -5396,7 +5399,7 @@
         <v/>
       </c>
       <c r="AA23">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G23/100,IF(Settings!$B$9,CEILING(MAX(0,V23+Settings!$B$2*G23/100-X23-Settings!$B$2*J23/100),Settings!$B$5),MAX(0,V23+Settings!$B$2*G23/100-X23-Settings!$B$2*J23/100))),IF(Settings!$B$9,MROUND(Z23,Settings!$B$5),Z23))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G23/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H23-I23+J23)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H23-I23+J23)/100))),IF(Settings!$B$9,MROUND(Z23,Settings!$B$5),Z23))</f>
         <v/>
       </c>
       <c r="AB23">
@@ -5513,7 +5516,7 @@
         <v/>
       </c>
       <c r="AA24">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G24/100,IF(Settings!$B$9,CEILING(MAX(0,V24+Settings!$B$2*G24/100-X24-Settings!$B$2*J24/100),Settings!$B$5),MAX(0,V24+Settings!$B$2*G24/100-X24-Settings!$B$2*J24/100))),IF(Settings!$B$9,MROUND(Z24,Settings!$B$5),Z24))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G24/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H24-I24+J24)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H24-I24+J24)/100))),IF(Settings!$B$9,MROUND(Z24,Settings!$B$5),Z24))</f>
         <v/>
       </c>
       <c r="AB24">
@@ -5630,7 +5633,7 @@
         <v/>
       </c>
       <c r="AA25">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G25/100,IF(Settings!$B$9,CEILING(MAX(0,V25+Settings!$B$2*G25/100-X25-Settings!$B$2*J25/100),Settings!$B$5),MAX(0,V25+Settings!$B$2*G25/100-X25-Settings!$B$2*J25/100))),IF(Settings!$B$9,MROUND(Z25,Settings!$B$5),Z25))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G25/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H25-I25+J25)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H25-I25+J25)/100))),IF(Settings!$B$9,MROUND(Z25,Settings!$B$5),Z25))</f>
         <v/>
       </c>
       <c r="AB25">
@@ -5747,7 +5750,7 @@
         <v/>
       </c>
       <c r="AA26">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G26/100,IF(Settings!$B$9,CEILING(MAX(0,V26+Settings!$B$2*G26/100-X26-Settings!$B$2*J26/100),Settings!$B$5),MAX(0,V26+Settings!$B$2*G26/100-X26-Settings!$B$2*J26/100))),IF(Settings!$B$9,MROUND(Z26,Settings!$B$5),Z26))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G26/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H26-I26+J26)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H26-I26+J26)/100))),IF(Settings!$B$9,MROUND(Z26,Settings!$B$5),Z26))</f>
         <v/>
       </c>
       <c r="AB26">
@@ -5864,7 +5867,7 @@
         <v/>
       </c>
       <c r="AA27">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G27/100,IF(Settings!$B$9,CEILING(MAX(0,V27+Settings!$B$2*G27/100-X27-Settings!$B$2*J27/100),Settings!$B$5),MAX(0,V27+Settings!$B$2*G27/100-X27-Settings!$B$2*J27/100))),IF(Settings!$B$9,MROUND(Z27,Settings!$B$5),Z27))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G27/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H27-I27+J27)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H27-I27+J27)/100))),IF(Settings!$B$9,MROUND(Z27,Settings!$B$5),Z27))</f>
         <v/>
       </c>
       <c r="AB27">
@@ -5981,7 +5984,7 @@
         <v/>
       </c>
       <c r="AA28">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G28/100,IF(Settings!$B$9,CEILING(MAX(0,V28+Settings!$B$2*G28/100-X28-Settings!$B$2*J28/100),Settings!$B$5),MAX(0,V28+Settings!$B$2*G28/100-X28-Settings!$B$2*J28/100))),IF(Settings!$B$9,MROUND(Z28,Settings!$B$5),Z28))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G28/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H28-I28+J28)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H28-I28+J28)/100))),IF(Settings!$B$9,MROUND(Z28,Settings!$B$5),Z28))</f>
         <v/>
       </c>
       <c r="AB28">
@@ -6098,7 +6101,7 @@
         <v/>
       </c>
       <c r="AA29">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G29/100,IF(Settings!$B$9,CEILING(MAX(0,V29+Settings!$B$2*G29/100-X29-Settings!$B$2*J29/100),Settings!$B$5),MAX(0,V29+Settings!$B$2*G29/100-X29-Settings!$B$2*J29/100))),IF(Settings!$B$9,MROUND(Z29,Settings!$B$5),Z29))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G29/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H29-I29+J29)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H29-I29+J29)/100))),IF(Settings!$B$9,MROUND(Z29,Settings!$B$5),Z29))</f>
         <v/>
       </c>
       <c r="AB29">
@@ -6215,7 +6218,7 @@
         <v/>
       </c>
       <c r="AA30">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G30/100,IF(Settings!$B$9,CEILING(MAX(0,V30+Settings!$B$2*G30/100-X30-Settings!$B$2*J30/100),Settings!$B$5),MAX(0,V30+Settings!$B$2*G30/100-X30-Settings!$B$2*J30/100))),IF(Settings!$B$9,MROUND(Z30,Settings!$B$5),Z30))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G30/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H30-I30+J30)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H30-I30+J30)/100))),IF(Settings!$B$9,MROUND(Z30,Settings!$B$5),Z30))</f>
         <v/>
       </c>
       <c r="AB30">
@@ -6332,7 +6335,7 @@
         <v/>
       </c>
       <c r="AA31">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G31/100,IF(Settings!$B$9,CEILING(MAX(0,V31+Settings!$B$2*G31/100-X31-Settings!$B$2*J31/100),Settings!$B$5),MAX(0,V31+Settings!$B$2*G31/100-X31-Settings!$B$2*J31/100))),IF(Settings!$B$9,MROUND(Z31,Settings!$B$5),Z31))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G31/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H31-I31+J31)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H31-I31+J31)/100))),IF(Settings!$B$9,MROUND(Z31,Settings!$B$5),Z31))</f>
         <v/>
       </c>
       <c r="AB31">
@@ -6449,7 +6452,7 @@
         <v/>
       </c>
       <c r="AA32">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G32/100,IF(Settings!$B$9,CEILING(MAX(0,V32+Settings!$B$2*G32/100-X32-Settings!$B$2*J32/100),Settings!$B$5),MAX(0,V32+Settings!$B$2*G32/100-X32-Settings!$B$2*J32/100))),IF(Settings!$B$9,MROUND(Z32,Settings!$B$5),Z32))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G32/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H32-I32+J32)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H32-I32+J32)/100))),IF(Settings!$B$9,MROUND(Z32,Settings!$B$5),Z32))</f>
         <v/>
       </c>
       <c r="AB32">
@@ -6566,7 +6569,7 @@
         <v/>
       </c>
       <c r="AA33">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G33/100,IF(Settings!$B$9,CEILING(MAX(0,V33+Settings!$B$2*G33/100-X33-Settings!$B$2*J33/100),Settings!$B$5),MAX(0,V33+Settings!$B$2*G33/100-X33-Settings!$B$2*J33/100))),IF(Settings!$B$9,MROUND(Z33,Settings!$B$5),Z33))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G33/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H33-I33+J33)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H33-I33+J33)/100))),IF(Settings!$B$9,MROUND(Z33,Settings!$B$5),Z33))</f>
         <v/>
       </c>
       <c r="AB33">
@@ -6683,7 +6686,7 @@
         <v/>
       </c>
       <c r="AA34">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G34/100,IF(Settings!$B$9,CEILING(MAX(0,V34+Settings!$B$2*G34/100-X34-Settings!$B$2*J34/100),Settings!$B$5),MAX(0,V34+Settings!$B$2*G34/100-X34-Settings!$B$2*J34/100))),IF(Settings!$B$9,MROUND(Z34,Settings!$B$5),Z34))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G34/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H34-I34+J34)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H34-I34+J34)/100))),IF(Settings!$B$9,MROUND(Z34,Settings!$B$5),Z34))</f>
         <v/>
       </c>
       <c r="AB34">
@@ -6800,7 +6803,7 @@
         <v/>
       </c>
       <c r="AA35">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G35/100,IF(Settings!$B$9,CEILING(MAX(0,V35+Settings!$B$2*G35/100-X35-Settings!$B$2*J35/100),Settings!$B$5),MAX(0,V35+Settings!$B$2*G35/100-X35-Settings!$B$2*J35/100))),IF(Settings!$B$9,MROUND(Z35,Settings!$B$5),Z35))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G35/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H35-I35+J35)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H35-I35+J35)/100))),IF(Settings!$B$9,MROUND(Z35,Settings!$B$5),Z35))</f>
         <v/>
       </c>
       <c r="AB35">
@@ -6917,7 +6920,7 @@
         <v/>
       </c>
       <c r="AA36">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G36/100,IF(Settings!$B$9,CEILING(MAX(0,V36+Settings!$B$2*G36/100-X36-Settings!$B$2*J36/100),Settings!$B$5),MAX(0,V36+Settings!$B$2*G36/100-X36-Settings!$B$2*J36/100))),IF(Settings!$B$9,MROUND(Z36,Settings!$B$5),Z36))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G36/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H36-I36+J36)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H36-I36+J36)/100))),IF(Settings!$B$9,MROUND(Z36,Settings!$B$5),Z36))</f>
         <v/>
       </c>
       <c r="AB36">
@@ -7034,7 +7037,7 @@
         <v/>
       </c>
       <c r="AA37">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G37/100,IF(Settings!$B$9,CEILING(MAX(0,V37+Settings!$B$2*G37/100-X37-Settings!$B$2*J37/100),Settings!$B$5),MAX(0,V37+Settings!$B$2*G37/100-X37-Settings!$B$2*J37/100))),IF(Settings!$B$9,MROUND(Z37,Settings!$B$5),Z37))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G37/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H37-I37+J37)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H37-I37+J37)/100))),IF(Settings!$B$9,MROUND(Z37,Settings!$B$5),Z37))</f>
         <v/>
       </c>
       <c r="AB37">
@@ -7151,7 +7154,7 @@
         <v/>
       </c>
       <c r="AA38">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G38/100,IF(Settings!$B$9,CEILING(MAX(0,V38+Settings!$B$2*G38/100-X38-Settings!$B$2*J38/100),Settings!$B$5),MAX(0,V38+Settings!$B$2*G38/100-X38-Settings!$B$2*J38/100))),IF(Settings!$B$9,MROUND(Z38,Settings!$B$5),Z38))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G38/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H38-I38+J38)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H38-I38+J38)/100))),IF(Settings!$B$9,MROUND(Z38,Settings!$B$5),Z38))</f>
         <v/>
       </c>
       <c r="AB38">
@@ -7268,7 +7271,7 @@
         <v/>
       </c>
       <c r="AA39">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G39/100,IF(Settings!$B$9,CEILING(MAX(0,V39+Settings!$B$2*G39/100-X39-Settings!$B$2*J39/100),Settings!$B$5),MAX(0,V39+Settings!$B$2*G39/100-X39-Settings!$B$2*J39/100))),IF(Settings!$B$9,MROUND(Z39,Settings!$B$5),Z39))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G39/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H39-I39+J39)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H39-I39+J39)/100))),IF(Settings!$B$9,MROUND(Z39,Settings!$B$5),Z39))</f>
         <v/>
       </c>
       <c r="AB39">
@@ -7385,7 +7388,7 @@
         <v/>
       </c>
       <c r="AA40">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G40/100,IF(Settings!$B$9,CEILING(MAX(0,V40+Settings!$B$2*G40/100-X40-Settings!$B$2*J40/100),Settings!$B$5),MAX(0,V40+Settings!$B$2*G40/100-X40-Settings!$B$2*J40/100))),IF(Settings!$B$9,MROUND(Z40,Settings!$B$5),Z40))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G40/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H40-I40+J40)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H40-I40+J40)/100))),IF(Settings!$B$9,MROUND(Z40,Settings!$B$5),Z40))</f>
         <v/>
       </c>
       <c r="AB40">
@@ -7502,7 +7505,7 @@
         <v/>
       </c>
       <c r="AA41">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G41/100,IF(Settings!$B$9,CEILING(MAX(0,V41+Settings!$B$2*G41/100-X41-Settings!$B$2*J41/100),Settings!$B$5),MAX(0,V41+Settings!$B$2*G41/100-X41-Settings!$B$2*J41/100))),IF(Settings!$B$9,MROUND(Z41,Settings!$B$5),Z41))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G41/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H41-I41+J41)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H41-I41+J41)/100))),IF(Settings!$B$9,MROUND(Z41,Settings!$B$5),Z41))</f>
         <v/>
       </c>
       <c r="AB41">
@@ -7889,7 +7892,7 @@
         <v/>
       </c>
       <c r="AA3">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G3/100,IF(Settings!$B$9,CEILING(MAX(0,V3+Settings!$B$2*G3/100-X3-Settings!$B$2*J3/100),Settings!$B$5),MAX(0,V3+Settings!$B$2*G3/100-X3-Settings!$B$2*J3/100))),IF(Settings!$B$9,MROUND(Z3,Settings!$B$5),Z3))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G3/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H3-I3+J3)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H3-I3+J3)/100))),IF(Settings!$B$9,MROUND(Z3,Settings!$B$5),Z3))</f>
         <v/>
       </c>
       <c r="AB3">
@@ -8006,7 +8009,7 @@
         <v/>
       </c>
       <c r="AA4">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G4/100,IF(Settings!$B$9,CEILING(MAX(0,V4+Settings!$B$2*G4/100-X4-Settings!$B$2*J4/100),Settings!$B$5),MAX(0,V4+Settings!$B$2*G4/100-X4-Settings!$B$2*J4/100))),IF(Settings!$B$9,MROUND(Z4,Settings!$B$5),Z4))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G4/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H4-I4+J4)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H4-I4+J4)/100))),IF(Settings!$B$9,MROUND(Z4,Settings!$B$5),Z4))</f>
         <v/>
       </c>
       <c r="AB4">
@@ -8123,7 +8126,7 @@
         <v/>
       </c>
       <c r="AA5">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G5/100,IF(Settings!$B$9,CEILING(MAX(0,V5+Settings!$B$2*G5/100-X5-Settings!$B$2*J5/100),Settings!$B$5),MAX(0,V5+Settings!$B$2*G5/100-X5-Settings!$B$2*J5/100))),IF(Settings!$B$9,MROUND(Z5,Settings!$B$5),Z5))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G5/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H5-I5+J5)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H5-I5+J5)/100))),IF(Settings!$B$9,MROUND(Z5,Settings!$B$5),Z5))</f>
         <v/>
       </c>
       <c r="AB5">
@@ -8240,7 +8243,7 @@
         <v/>
       </c>
       <c r="AA6">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G6/100,IF(Settings!$B$9,CEILING(MAX(0,V6+Settings!$B$2*G6/100-X6-Settings!$B$2*J6/100),Settings!$B$5),MAX(0,V6+Settings!$B$2*G6/100-X6-Settings!$B$2*J6/100))),IF(Settings!$B$9,MROUND(Z6,Settings!$B$5),Z6))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G6/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H6-I6+J6)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H6-I6+J6)/100))),IF(Settings!$B$9,MROUND(Z6,Settings!$B$5),Z6))</f>
         <v/>
       </c>
       <c r="AB6">
@@ -8357,7 +8360,7 @@
         <v/>
       </c>
       <c r="AA7">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G7/100,IF(Settings!$B$9,CEILING(MAX(0,V7+Settings!$B$2*G7/100-X7-Settings!$B$2*J7/100),Settings!$B$5),MAX(0,V7+Settings!$B$2*G7/100-X7-Settings!$B$2*J7/100))),IF(Settings!$B$9,MROUND(Z7,Settings!$B$5),Z7))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G7/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H7-I7+J7)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H7-I7+J7)/100))),IF(Settings!$B$9,MROUND(Z7,Settings!$B$5),Z7))</f>
         <v/>
       </c>
       <c r="AB7">
@@ -8474,7 +8477,7 @@
         <v/>
       </c>
       <c r="AA8">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G8/100,IF(Settings!$B$9,CEILING(MAX(0,V8+Settings!$B$2*G8/100-X8-Settings!$B$2*J8/100),Settings!$B$5),MAX(0,V8+Settings!$B$2*G8/100-X8-Settings!$B$2*J8/100))),IF(Settings!$B$9,MROUND(Z8,Settings!$B$5),Z8))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G8/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H8-I8+J8)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H8-I8+J8)/100))),IF(Settings!$B$9,MROUND(Z8,Settings!$B$5),Z8))</f>
         <v/>
       </c>
       <c r="AB8">
@@ -8591,7 +8594,7 @@
         <v/>
       </c>
       <c r="AA9">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G9/100,IF(Settings!$B$9,CEILING(MAX(0,V9+Settings!$B$2*G9/100-X9-Settings!$B$2*J9/100),Settings!$B$5),MAX(0,V9+Settings!$B$2*G9/100-X9-Settings!$B$2*J9/100))),IF(Settings!$B$9,MROUND(Z9,Settings!$B$5),Z9))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G9/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H9-I9+J9)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H9-I9+J9)/100))),IF(Settings!$B$9,MROUND(Z9,Settings!$B$5),Z9))</f>
         <v/>
       </c>
       <c r="AB9">
@@ -8708,7 +8711,7 @@
         <v/>
       </c>
       <c r="AA10">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G10/100,IF(Settings!$B$9,CEILING(MAX(0,V10+Settings!$B$2*G10/100-X10-Settings!$B$2*J10/100),Settings!$B$5),MAX(0,V10+Settings!$B$2*G10/100-X10-Settings!$B$2*J10/100))),IF(Settings!$B$9,MROUND(Z10,Settings!$B$5),Z10))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G10/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H10-I10+J10)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H10-I10+J10)/100))),IF(Settings!$B$9,MROUND(Z10,Settings!$B$5),Z10))</f>
         <v/>
       </c>
       <c r="AB10">
@@ -8825,7 +8828,7 @@
         <v/>
       </c>
       <c r="AA11">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G11/100,IF(Settings!$B$9,CEILING(MAX(0,V11+Settings!$B$2*G11/100-X11-Settings!$B$2*J11/100),Settings!$B$5),MAX(0,V11+Settings!$B$2*G11/100-X11-Settings!$B$2*J11/100))),IF(Settings!$B$9,MROUND(Z11,Settings!$B$5),Z11))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G11/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H11-I11+J11)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H11-I11+J11)/100))),IF(Settings!$B$9,MROUND(Z11,Settings!$B$5),Z11))</f>
         <v/>
       </c>
       <c r="AB11">
@@ -8942,7 +8945,7 @@
         <v/>
       </c>
       <c r="AA12">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G12/100,IF(Settings!$B$9,CEILING(MAX(0,V12+Settings!$B$2*G12/100-X12-Settings!$B$2*J12/100),Settings!$B$5),MAX(0,V12+Settings!$B$2*G12/100-X12-Settings!$B$2*J12/100))),IF(Settings!$B$9,MROUND(Z12,Settings!$B$5),Z12))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G12/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H12-I12+J12)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H12-I12+J12)/100))),IF(Settings!$B$9,MROUND(Z12,Settings!$B$5),Z12))</f>
         <v/>
       </c>
       <c r="AB12">
@@ -9059,7 +9062,7 @@
         <v/>
       </c>
       <c r="AA13">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G13/100,IF(Settings!$B$9,CEILING(MAX(0,V13+Settings!$B$2*G13/100-X13-Settings!$B$2*J13/100),Settings!$B$5),MAX(0,V13+Settings!$B$2*G13/100-X13-Settings!$B$2*J13/100))),IF(Settings!$B$9,MROUND(Z13,Settings!$B$5),Z13))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G13/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H13-I13+J13)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H13-I13+J13)/100))),IF(Settings!$B$9,MROUND(Z13,Settings!$B$5),Z13))</f>
         <v/>
       </c>
       <c r="AB13">
@@ -9176,7 +9179,7 @@
         <v/>
       </c>
       <c r="AA14">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G14/100,IF(Settings!$B$9,CEILING(MAX(0,V14+Settings!$B$2*G14/100-X14-Settings!$B$2*J14/100),Settings!$B$5),MAX(0,V14+Settings!$B$2*G14/100-X14-Settings!$B$2*J14/100))),IF(Settings!$B$9,MROUND(Z14,Settings!$B$5),Z14))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G14/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H14-I14+J14)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H14-I14+J14)/100))),IF(Settings!$B$9,MROUND(Z14,Settings!$B$5),Z14))</f>
         <v/>
       </c>
       <c r="AB14">
@@ -9293,7 +9296,7 @@
         <v/>
       </c>
       <c r="AA15">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G15/100,IF(Settings!$B$9,CEILING(MAX(0,V15+Settings!$B$2*G15/100-X15-Settings!$B$2*J15/100),Settings!$B$5),MAX(0,V15+Settings!$B$2*G15/100-X15-Settings!$B$2*J15/100))),IF(Settings!$B$9,MROUND(Z15,Settings!$B$5),Z15))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G15/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H15-I15+J15)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H15-I15+J15)/100))),IF(Settings!$B$9,MROUND(Z15,Settings!$B$5),Z15))</f>
         <v/>
       </c>
       <c r="AB15">
@@ -9410,7 +9413,7 @@
         <v/>
       </c>
       <c r="AA16">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G16/100,IF(Settings!$B$9,CEILING(MAX(0,V16+Settings!$B$2*G16/100-X16-Settings!$B$2*J16/100),Settings!$B$5),MAX(0,V16+Settings!$B$2*G16/100-X16-Settings!$B$2*J16/100))),IF(Settings!$B$9,MROUND(Z16,Settings!$B$5),Z16))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G16/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H16-I16+J16)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H16-I16+J16)/100))),IF(Settings!$B$9,MROUND(Z16,Settings!$B$5),Z16))</f>
         <v/>
       </c>
       <c r="AB16">
@@ -9527,7 +9530,7 @@
         <v/>
       </c>
       <c r="AA17">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G17/100,IF(Settings!$B$9,CEILING(MAX(0,V17+Settings!$B$2*G17/100-X17-Settings!$B$2*J17/100),Settings!$B$5),MAX(0,V17+Settings!$B$2*G17/100-X17-Settings!$B$2*J17/100))),IF(Settings!$B$9,MROUND(Z17,Settings!$B$5),Z17))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G17/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H17-I17+J17)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H17-I17+J17)/100))),IF(Settings!$B$9,MROUND(Z17,Settings!$B$5),Z17))</f>
         <v/>
       </c>
       <c r="AB17">
@@ -9644,7 +9647,7 @@
         <v/>
       </c>
       <c r="AA18">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G18/100,IF(Settings!$B$9,CEILING(MAX(0,V18+Settings!$B$2*G18/100-X18-Settings!$B$2*J18/100),Settings!$B$5),MAX(0,V18+Settings!$B$2*G18/100-X18-Settings!$B$2*J18/100))),IF(Settings!$B$9,MROUND(Z18,Settings!$B$5),Z18))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G18/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H18-I18+J18)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H18-I18+J18)/100))),IF(Settings!$B$9,MROUND(Z18,Settings!$B$5),Z18))</f>
         <v/>
       </c>
       <c r="AB18">
@@ -9761,7 +9764,7 @@
         <v/>
       </c>
       <c r="AA19">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G19/100,IF(Settings!$B$9,CEILING(MAX(0,V19+Settings!$B$2*G19/100-X19-Settings!$B$2*J19/100),Settings!$B$5),MAX(0,V19+Settings!$B$2*G19/100-X19-Settings!$B$2*J19/100))),IF(Settings!$B$9,MROUND(Z19,Settings!$B$5),Z19))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G19/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H19-I19+J19)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H19-I19+J19)/100))),IF(Settings!$B$9,MROUND(Z19,Settings!$B$5),Z19))</f>
         <v/>
       </c>
       <c r="AB19">
@@ -9878,7 +9881,7 @@
         <v/>
       </c>
       <c r="AA20">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G20/100,IF(Settings!$B$9,CEILING(MAX(0,V20+Settings!$B$2*G20/100-X20-Settings!$B$2*J20/100),Settings!$B$5),MAX(0,V20+Settings!$B$2*G20/100-X20-Settings!$B$2*J20/100))),IF(Settings!$B$9,MROUND(Z20,Settings!$B$5),Z20))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G20/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H20-I20+J20)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H20-I20+J20)/100))),IF(Settings!$B$9,MROUND(Z20,Settings!$B$5),Z20))</f>
         <v/>
       </c>
       <c r="AB20">
@@ -9995,7 +9998,7 @@
         <v/>
       </c>
       <c r="AA21">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G21/100,IF(Settings!$B$9,CEILING(MAX(0,V21+Settings!$B$2*G21/100-X21-Settings!$B$2*J21/100),Settings!$B$5),MAX(0,V21+Settings!$B$2*G21/100-X21-Settings!$B$2*J21/100))),IF(Settings!$B$9,MROUND(Z21,Settings!$B$5),Z21))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G21/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H21-I21+J21)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H21-I21+J21)/100))),IF(Settings!$B$9,MROUND(Z21,Settings!$B$5),Z21))</f>
         <v/>
       </c>
       <c r="AB21">
@@ -10112,7 +10115,7 @@
         <v/>
       </c>
       <c r="AA22">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G22/100,IF(Settings!$B$9,CEILING(MAX(0,V22+Settings!$B$2*G22/100-X22-Settings!$B$2*J22/100),Settings!$B$5),MAX(0,V22+Settings!$B$2*G22/100-X22-Settings!$B$2*J22/100))),IF(Settings!$B$9,MROUND(Z22,Settings!$B$5),Z22))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G22/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H22-I22+J22)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H22-I22+J22)/100))),IF(Settings!$B$9,MROUND(Z22,Settings!$B$5),Z22))</f>
         <v/>
       </c>
       <c r="AB22">
@@ -10229,7 +10232,7 @@
         <v/>
       </c>
       <c r="AA23">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G23/100,IF(Settings!$B$9,CEILING(MAX(0,V23+Settings!$B$2*G23/100-X23-Settings!$B$2*J23/100),Settings!$B$5),MAX(0,V23+Settings!$B$2*G23/100-X23-Settings!$B$2*J23/100))),IF(Settings!$B$9,MROUND(Z23,Settings!$B$5),Z23))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G23/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H23-I23+J23)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H23-I23+J23)/100))),IF(Settings!$B$9,MROUND(Z23,Settings!$B$5),Z23))</f>
         <v/>
       </c>
       <c r="AB23">
@@ -10346,7 +10349,7 @@
         <v/>
       </c>
       <c r="AA24">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G24/100,IF(Settings!$B$9,CEILING(MAX(0,V24+Settings!$B$2*G24/100-X24-Settings!$B$2*J24/100),Settings!$B$5),MAX(0,V24+Settings!$B$2*G24/100-X24-Settings!$B$2*J24/100))),IF(Settings!$B$9,MROUND(Z24,Settings!$B$5),Z24))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G24/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H24-I24+J24)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H24-I24+J24)/100))),IF(Settings!$B$9,MROUND(Z24,Settings!$B$5),Z24))</f>
         <v/>
       </c>
       <c r="AB24">
@@ -10463,7 +10466,7 @@
         <v/>
       </c>
       <c r="AA25">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G25/100,IF(Settings!$B$9,CEILING(MAX(0,V25+Settings!$B$2*G25/100-X25-Settings!$B$2*J25/100),Settings!$B$5),MAX(0,V25+Settings!$B$2*G25/100-X25-Settings!$B$2*J25/100))),IF(Settings!$B$9,MROUND(Z25,Settings!$B$5),Z25))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G25/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H25-I25+J25)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H25-I25+J25)/100))),IF(Settings!$B$9,MROUND(Z25,Settings!$B$5),Z25))</f>
         <v/>
       </c>
       <c r="AB25">
@@ -10580,7 +10583,7 @@
         <v/>
       </c>
       <c r="AA26">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G26/100,IF(Settings!$B$9,CEILING(MAX(0,V26+Settings!$B$2*G26/100-X26-Settings!$B$2*J26/100),Settings!$B$5),MAX(0,V26+Settings!$B$2*G26/100-X26-Settings!$B$2*J26/100))),IF(Settings!$B$9,MROUND(Z26,Settings!$B$5),Z26))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G26/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H26-I26+J26)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H26-I26+J26)/100))),IF(Settings!$B$9,MROUND(Z26,Settings!$B$5),Z26))</f>
         <v/>
       </c>
       <c r="AB26">
@@ -10697,7 +10700,7 @@
         <v/>
       </c>
       <c r="AA27">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G27/100,IF(Settings!$B$9,CEILING(MAX(0,V27+Settings!$B$2*G27/100-X27-Settings!$B$2*J27/100),Settings!$B$5),MAX(0,V27+Settings!$B$2*G27/100-X27-Settings!$B$2*J27/100))),IF(Settings!$B$9,MROUND(Z27,Settings!$B$5),Z27))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G27/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H27-I27+J27)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H27-I27+J27)/100))),IF(Settings!$B$9,MROUND(Z27,Settings!$B$5),Z27))</f>
         <v/>
       </c>
       <c r="AB27">
@@ -10814,7 +10817,7 @@
         <v/>
       </c>
       <c r="AA28">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G28/100,IF(Settings!$B$9,CEILING(MAX(0,V28+Settings!$B$2*G28/100-X28-Settings!$B$2*J28/100),Settings!$B$5),MAX(0,V28+Settings!$B$2*G28/100-X28-Settings!$B$2*J28/100))),IF(Settings!$B$9,MROUND(Z28,Settings!$B$5),Z28))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G28/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H28-I28+J28)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H28-I28+J28)/100))),IF(Settings!$B$9,MROUND(Z28,Settings!$B$5),Z28))</f>
         <v/>
       </c>
       <c r="AB28">
@@ -10931,7 +10934,7 @@
         <v/>
       </c>
       <c r="AA29">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G29/100,IF(Settings!$B$9,CEILING(MAX(0,V29+Settings!$B$2*G29/100-X29-Settings!$B$2*J29/100),Settings!$B$5),MAX(0,V29+Settings!$B$2*G29/100-X29-Settings!$B$2*J29/100))),IF(Settings!$B$9,MROUND(Z29,Settings!$B$5),Z29))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G29/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H29-I29+J29)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H29-I29+J29)/100))),IF(Settings!$B$9,MROUND(Z29,Settings!$B$5),Z29))</f>
         <v/>
       </c>
       <c r="AB29">
@@ -11048,7 +11051,7 @@
         <v/>
       </c>
       <c r="AA30">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G30/100,IF(Settings!$B$9,CEILING(MAX(0,V30+Settings!$B$2*G30/100-X30-Settings!$B$2*J30/100),Settings!$B$5),MAX(0,V30+Settings!$B$2*G30/100-X30-Settings!$B$2*J30/100))),IF(Settings!$B$9,MROUND(Z30,Settings!$B$5),Z30))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G30/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H30-I30+J30)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H30-I30+J30)/100))),IF(Settings!$B$9,MROUND(Z30,Settings!$B$5),Z30))</f>
         <v/>
       </c>
       <c r="AB30">
@@ -11165,7 +11168,7 @@
         <v/>
       </c>
       <c r="AA31">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G31/100,IF(Settings!$B$9,CEILING(MAX(0,V31+Settings!$B$2*G31/100-X31-Settings!$B$2*J31/100),Settings!$B$5),MAX(0,V31+Settings!$B$2*G31/100-X31-Settings!$B$2*J31/100))),IF(Settings!$B$9,MROUND(Z31,Settings!$B$5),Z31))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G31/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H31-I31+J31)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H31-I31+J31)/100))),IF(Settings!$B$9,MROUND(Z31,Settings!$B$5),Z31))</f>
         <v/>
       </c>
       <c r="AB31">
@@ -11282,7 +11285,7 @@
         <v/>
       </c>
       <c r="AA32">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G32/100,IF(Settings!$B$9,CEILING(MAX(0,V32+Settings!$B$2*G32/100-X32-Settings!$B$2*J32/100),Settings!$B$5),MAX(0,V32+Settings!$B$2*G32/100-X32-Settings!$B$2*J32/100))),IF(Settings!$B$9,MROUND(Z32,Settings!$B$5),Z32))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G32/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H32-I32+J32)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H32-I32+J32)/100))),IF(Settings!$B$9,MROUND(Z32,Settings!$B$5),Z32))</f>
         <v/>
       </c>
       <c r="AB32">
@@ -11399,7 +11402,7 @@
         <v/>
       </c>
       <c r="AA33">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G33/100,IF(Settings!$B$9,CEILING(MAX(0,V33+Settings!$B$2*G33/100-X33-Settings!$B$2*J33/100),Settings!$B$5),MAX(0,V33+Settings!$B$2*G33/100-X33-Settings!$B$2*J33/100))),IF(Settings!$B$9,MROUND(Z33,Settings!$B$5),Z33))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G33/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H33-I33+J33)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H33-I33+J33)/100))),IF(Settings!$B$9,MROUND(Z33,Settings!$B$5),Z33))</f>
         <v/>
       </c>
       <c r="AB33">
@@ -11516,7 +11519,7 @@
         <v/>
       </c>
       <c r="AA34">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G34/100,IF(Settings!$B$9,CEILING(MAX(0,V34+Settings!$B$2*G34/100-X34-Settings!$B$2*J34/100),Settings!$B$5),MAX(0,V34+Settings!$B$2*G34/100-X34-Settings!$B$2*J34/100))),IF(Settings!$B$9,MROUND(Z34,Settings!$B$5),Z34))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G34/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H34-I34+J34)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H34-I34+J34)/100))),IF(Settings!$B$9,MROUND(Z34,Settings!$B$5),Z34))</f>
         <v/>
       </c>
       <c r="AB34">
@@ -11633,7 +11636,7 @@
         <v/>
       </c>
       <c r="AA35">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G35/100,IF(Settings!$B$9,CEILING(MAX(0,V35+Settings!$B$2*G35/100-X35-Settings!$B$2*J35/100),Settings!$B$5),MAX(0,V35+Settings!$B$2*G35/100-X35-Settings!$B$2*J35/100))),IF(Settings!$B$9,MROUND(Z35,Settings!$B$5),Z35))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G35/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H35-I35+J35)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H35-I35+J35)/100))),IF(Settings!$B$9,MROUND(Z35,Settings!$B$5),Z35))</f>
         <v/>
       </c>
       <c r="AB35">
@@ -11750,7 +11753,7 @@
         <v/>
       </c>
       <c r="AA36">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G36/100,IF(Settings!$B$9,CEILING(MAX(0,V36+Settings!$B$2*G36/100-X36-Settings!$B$2*J36/100),Settings!$B$5),MAX(0,V36+Settings!$B$2*G36/100-X36-Settings!$B$2*J36/100))),IF(Settings!$B$9,MROUND(Z36,Settings!$B$5),Z36))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G36/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H36-I36+J36)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H36-I36+J36)/100))),IF(Settings!$B$9,MROUND(Z36,Settings!$B$5),Z36))</f>
         <v/>
       </c>
       <c r="AB36">
@@ -11867,7 +11870,7 @@
         <v/>
       </c>
       <c r="AA37">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G37/100,IF(Settings!$B$9,CEILING(MAX(0,V37+Settings!$B$2*G37/100-X37-Settings!$B$2*J37/100),Settings!$B$5),MAX(0,V37+Settings!$B$2*G37/100-X37-Settings!$B$2*J37/100))),IF(Settings!$B$9,MROUND(Z37,Settings!$B$5),Z37))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G37/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H37-I37+J37)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H37-I37+J37)/100))),IF(Settings!$B$9,MROUND(Z37,Settings!$B$5),Z37))</f>
         <v/>
       </c>
       <c r="AB37">
@@ -11984,7 +11987,7 @@
         <v/>
       </c>
       <c r="AA38">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G38/100,IF(Settings!$B$9,CEILING(MAX(0,V38+Settings!$B$2*G38/100-X38-Settings!$B$2*J38/100),Settings!$B$5),MAX(0,V38+Settings!$B$2*G38/100-X38-Settings!$B$2*J38/100))),IF(Settings!$B$9,MROUND(Z38,Settings!$B$5),Z38))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G38/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H38-I38+J38)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H38-I38+J38)/100))),IF(Settings!$B$9,MROUND(Z38,Settings!$B$5),Z38))</f>
         <v/>
       </c>
       <c r="AB38">
@@ -12101,7 +12104,7 @@
         <v/>
       </c>
       <c r="AA39">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G39/100,IF(Settings!$B$9,CEILING(MAX(0,V39+Settings!$B$2*G39/100-X39-Settings!$B$2*J39/100),Settings!$B$5),MAX(0,V39+Settings!$B$2*G39/100-X39-Settings!$B$2*J39/100))),IF(Settings!$B$9,MROUND(Z39,Settings!$B$5),Z39))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G39/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H39-I39+J39)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H39-I39+J39)/100))),IF(Settings!$B$9,MROUND(Z39,Settings!$B$5),Z39))</f>
         <v/>
       </c>
       <c r="AB39">
@@ -12218,7 +12221,7 @@
         <v/>
       </c>
       <c r="AA40">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G40/100,IF(Settings!$B$9,CEILING(MAX(0,V40+Settings!$B$2*G40/100-X40-Settings!$B$2*J40/100),Settings!$B$5),MAX(0,V40+Settings!$B$2*G40/100-X40-Settings!$B$2*J40/100))),IF(Settings!$B$9,MROUND(Z40,Settings!$B$5),Z40))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G40/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H40-I40+J40)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H40-I40+J40)/100))),IF(Settings!$B$9,MROUND(Z40,Settings!$B$5),Z40))</f>
         <v/>
       </c>
       <c r="AB40">
@@ -12335,7 +12338,7 @@
         <v/>
       </c>
       <c r="AA41">
-        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G41/100,IF(Settings!$B$9,CEILING(MAX(0,V41+Settings!$B$2*G41/100-X41-Settings!$B$2*J41/100),Settings!$B$5),MAX(0,V41+Settings!$B$2*G41/100-X41-Settings!$B$2*J41/100))),IF(Settings!$B$9,MROUND(Z41,Settings!$B$5),Z41))</f>
+        <f>IF(Settings!$B$17,MIN(Settings!$B$2*G41/100,IF(Settings!$B$9,CEILING(MAX(0,Settings!$B$2*(H41-I41+J41)/100),Settings!$B$5),MAX(0,Settings!$B$2*(H41-I41+J41)/100))),IF(Settings!$B$9,MROUND(Z41,Settings!$B$5),Z41))</f>
         <v/>
       </c>
       <c r="AB41">
@@ -12444,7 +12447,7 @@
         </is>
       </c>
       <c r="B8">
-        <f>RiskDashboard!B2</f>
+        <f>RiskDashboard!B4</f>
         <v/>
       </c>
     </row>
@@ -12466,7 +12469,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>RiskDashboard!B5</f>
+        <f>RiskDashboard!B7</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Finalize V3 rounded-risk validation and full system tests
</commit_message>
<xml_diff>
--- a/MinusLock_Percent_Grid_Calculator/MinusLock_Percent_Grid_Calculator.xlsx
+++ b/MinusLock_Percent_Grid_Calculator/MinusLock_Percent_Grid_Calculator.xlsx
@@ -2709,7 +2709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC41"/>
+  <dimension ref="A1:AJ41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2858,6 +2858,41 @@
           <t>Rounding Comment</t>
         </is>
       </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>Rounded Start After Lot</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Rounded Sum Big Lot</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Rounded Sum Small Lot</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Rounded Total Main Lot</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Rounded Total Opposite Lot</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>Rounded Skew Lot</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>Rounded Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -2954,6 +2989,27 @@
         <f>IF(AB2="FIXED","Close adjusted by SAFE mode",IF(AB2="SAFE","BUY/SELL balance preserved",IF(AB2="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -3070,6 +3126,34 @@
         <f>IF(AB3="FIXED","Close adjusted by SAFE mode",IF(AB3="SAFE","BUY/SELL balance preserved",IF(AB3="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD3">
+        <f>MAX(0,Settings!$B$2*G3/100-AA3)</f>
+        <v/>
+      </c>
+      <c r="AE3">
+        <f>SUM($W$3:W3)</f>
+        <v/>
+      </c>
+      <c r="AF3">
+        <f>SUM($Y$3:Y3)</f>
+        <v/>
+      </c>
+      <c r="AG3">
+        <f>AD3+AE3</f>
+        <v/>
+      </c>
+      <c r="AH3">
+        <f>Settings!$B$2+AF3</f>
+        <v/>
+      </c>
+      <c r="AI3">
+        <f>AH3-AG3</f>
+        <v/>
+      </c>
+      <c r="AJ3">
+        <f>IF(OR(AND(C3&gt;0,W3=0),AND(E3&gt;0,Y3=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG3&gt;AH3,"ERROR: Rounded balance broken",IF(AI3&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -3187,6 +3271,34 @@
         <f>IF(AB4="FIXED","Close adjusted by SAFE mode",IF(AB4="SAFE","BUY/SELL balance preserved",IF(AB4="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD4">
+        <f>MAX(0,Settings!$B$2*G4/100-AA4)</f>
+        <v/>
+      </c>
+      <c r="AE4">
+        <f>SUM($W$3:W4)</f>
+        <v/>
+      </c>
+      <c r="AF4">
+        <f>SUM($Y$3:Y4)</f>
+        <v/>
+      </c>
+      <c r="AG4">
+        <f>AD4+AE4</f>
+        <v/>
+      </c>
+      <c r="AH4">
+        <f>Settings!$B$2+AF4</f>
+        <v/>
+      </c>
+      <c r="AI4">
+        <f>AH4-AG4</f>
+        <v/>
+      </c>
+      <c r="AJ4">
+        <f>IF(OR(AND(C4&gt;0,W4=0),AND(E4&gt;0,Y4=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG4&gt;AH4,"ERROR: Rounded balance broken",IF(AI4&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -3304,6 +3416,34 @@
         <f>IF(AB5="FIXED","Close adjusted by SAFE mode",IF(AB5="SAFE","BUY/SELL balance preserved",IF(AB5="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD5">
+        <f>MAX(0,Settings!$B$2*G5/100-AA5)</f>
+        <v/>
+      </c>
+      <c r="AE5">
+        <f>SUM($W$3:W5)</f>
+        <v/>
+      </c>
+      <c r="AF5">
+        <f>SUM($Y$3:Y5)</f>
+        <v/>
+      </c>
+      <c r="AG5">
+        <f>AD5+AE5</f>
+        <v/>
+      </c>
+      <c r="AH5">
+        <f>Settings!$B$2+AF5</f>
+        <v/>
+      </c>
+      <c r="AI5">
+        <f>AH5-AG5</f>
+        <v/>
+      </c>
+      <c r="AJ5">
+        <f>IF(OR(AND(C5&gt;0,W5=0),AND(E5&gt;0,Y5=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG5&gt;AH5,"ERROR: Rounded balance broken",IF(AI5&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -3421,6 +3561,34 @@
         <f>IF(AB6="FIXED","Close adjusted by SAFE mode",IF(AB6="SAFE","BUY/SELL balance preserved",IF(AB6="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD6">
+        <f>MAX(0,Settings!$B$2*G6/100-AA6)</f>
+        <v/>
+      </c>
+      <c r="AE6">
+        <f>SUM($W$3:W6)</f>
+        <v/>
+      </c>
+      <c r="AF6">
+        <f>SUM($Y$3:Y6)</f>
+        <v/>
+      </c>
+      <c r="AG6">
+        <f>AD6+AE6</f>
+        <v/>
+      </c>
+      <c r="AH6">
+        <f>Settings!$B$2+AF6</f>
+        <v/>
+      </c>
+      <c r="AI6">
+        <f>AH6-AG6</f>
+        <v/>
+      </c>
+      <c r="AJ6">
+        <f>IF(OR(AND(C6&gt;0,W6=0),AND(E6&gt;0,Y6=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG6&gt;AH6,"ERROR: Rounded balance broken",IF(AI6&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -3538,6 +3706,34 @@
         <f>IF(AB7="FIXED","Close adjusted by SAFE mode",IF(AB7="SAFE","BUY/SELL balance preserved",IF(AB7="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD7">
+        <f>MAX(0,Settings!$B$2*G7/100-AA7)</f>
+        <v/>
+      </c>
+      <c r="AE7">
+        <f>SUM($W$3:W7)</f>
+        <v/>
+      </c>
+      <c r="AF7">
+        <f>SUM($Y$3:Y7)</f>
+        <v/>
+      </c>
+      <c r="AG7">
+        <f>AD7+AE7</f>
+        <v/>
+      </c>
+      <c r="AH7">
+        <f>Settings!$B$2+AF7</f>
+        <v/>
+      </c>
+      <c r="AI7">
+        <f>AH7-AG7</f>
+        <v/>
+      </c>
+      <c r="AJ7">
+        <f>IF(OR(AND(C7&gt;0,W7=0),AND(E7&gt;0,Y7=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG7&gt;AH7,"ERROR: Rounded balance broken",IF(AI7&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -3655,6 +3851,34 @@
         <f>IF(AB8="FIXED","Close adjusted by SAFE mode",IF(AB8="SAFE","BUY/SELL balance preserved",IF(AB8="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD8">
+        <f>MAX(0,Settings!$B$2*G8/100-AA8)</f>
+        <v/>
+      </c>
+      <c r="AE8">
+        <f>SUM($W$3:W8)</f>
+        <v/>
+      </c>
+      <c r="AF8">
+        <f>SUM($Y$3:Y8)</f>
+        <v/>
+      </c>
+      <c r="AG8">
+        <f>AD8+AE8</f>
+        <v/>
+      </c>
+      <c r="AH8">
+        <f>Settings!$B$2+AF8</f>
+        <v/>
+      </c>
+      <c r="AI8">
+        <f>AH8-AG8</f>
+        <v/>
+      </c>
+      <c r="AJ8">
+        <f>IF(OR(AND(C8&gt;0,W8=0),AND(E8&gt;0,Y8=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG8&gt;AH8,"ERROR: Rounded balance broken",IF(AI8&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -3772,6 +3996,34 @@
         <f>IF(AB9="FIXED","Close adjusted by SAFE mode",IF(AB9="SAFE","BUY/SELL balance preserved",IF(AB9="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD9">
+        <f>MAX(0,Settings!$B$2*G9/100-AA9)</f>
+        <v/>
+      </c>
+      <c r="AE9">
+        <f>SUM($W$3:W9)</f>
+        <v/>
+      </c>
+      <c r="AF9">
+        <f>SUM($Y$3:Y9)</f>
+        <v/>
+      </c>
+      <c r="AG9">
+        <f>AD9+AE9</f>
+        <v/>
+      </c>
+      <c r="AH9">
+        <f>Settings!$B$2+AF9</f>
+        <v/>
+      </c>
+      <c r="AI9">
+        <f>AH9-AG9</f>
+        <v/>
+      </c>
+      <c r="AJ9">
+        <f>IF(OR(AND(C9&gt;0,W9=0),AND(E9&gt;0,Y9=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG9&gt;AH9,"ERROR: Rounded balance broken",IF(AI9&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -3889,6 +4141,34 @@
         <f>IF(AB10="FIXED","Close adjusted by SAFE mode",IF(AB10="SAFE","BUY/SELL balance preserved",IF(AB10="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD10">
+        <f>MAX(0,Settings!$B$2*G10/100-AA10)</f>
+        <v/>
+      </c>
+      <c r="AE10">
+        <f>SUM($W$3:W10)</f>
+        <v/>
+      </c>
+      <c r="AF10">
+        <f>SUM($Y$3:Y10)</f>
+        <v/>
+      </c>
+      <c r="AG10">
+        <f>AD10+AE10</f>
+        <v/>
+      </c>
+      <c r="AH10">
+        <f>Settings!$B$2+AF10</f>
+        <v/>
+      </c>
+      <c r="AI10">
+        <f>AH10-AG10</f>
+        <v/>
+      </c>
+      <c r="AJ10">
+        <f>IF(OR(AND(C10&gt;0,W10=0),AND(E10&gt;0,Y10=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG10&gt;AH10,"ERROR: Rounded balance broken",IF(AI10&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -4006,6 +4286,34 @@
         <f>IF(AB11="FIXED","Close adjusted by SAFE mode",IF(AB11="SAFE","BUY/SELL balance preserved",IF(AB11="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD11">
+        <f>MAX(0,Settings!$B$2*G11/100-AA11)</f>
+        <v/>
+      </c>
+      <c r="AE11">
+        <f>SUM($W$3:W11)</f>
+        <v/>
+      </c>
+      <c r="AF11">
+        <f>SUM($Y$3:Y11)</f>
+        <v/>
+      </c>
+      <c r="AG11">
+        <f>AD11+AE11</f>
+        <v/>
+      </c>
+      <c r="AH11">
+        <f>Settings!$B$2+AF11</f>
+        <v/>
+      </c>
+      <c r="AI11">
+        <f>AH11-AG11</f>
+        <v/>
+      </c>
+      <c r="AJ11">
+        <f>IF(OR(AND(C11&gt;0,W11=0),AND(E11&gt;0,Y11=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG11&gt;AH11,"ERROR: Rounded balance broken",IF(AI11&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -4123,6 +4431,34 @@
         <f>IF(AB12="FIXED","Close adjusted by SAFE mode",IF(AB12="SAFE","BUY/SELL balance preserved",IF(AB12="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD12">
+        <f>MAX(0,Settings!$B$2*G12/100-AA12)</f>
+        <v/>
+      </c>
+      <c r="AE12">
+        <f>SUM($W$3:W12)</f>
+        <v/>
+      </c>
+      <c r="AF12">
+        <f>SUM($Y$3:Y12)</f>
+        <v/>
+      </c>
+      <c r="AG12">
+        <f>AD12+AE12</f>
+        <v/>
+      </c>
+      <c r="AH12">
+        <f>Settings!$B$2+AF12</f>
+        <v/>
+      </c>
+      <c r="AI12">
+        <f>AH12-AG12</f>
+        <v/>
+      </c>
+      <c r="AJ12">
+        <f>IF(OR(AND(C12&gt;0,W12=0),AND(E12&gt;0,Y12=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG12&gt;AH12,"ERROR: Rounded balance broken",IF(AI12&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -4240,6 +4576,34 @@
         <f>IF(AB13="FIXED","Close adjusted by SAFE mode",IF(AB13="SAFE","BUY/SELL balance preserved",IF(AB13="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD13">
+        <f>MAX(0,Settings!$B$2*G13/100-AA13)</f>
+        <v/>
+      </c>
+      <c r="AE13">
+        <f>SUM($W$3:W13)</f>
+        <v/>
+      </c>
+      <c r="AF13">
+        <f>SUM($Y$3:Y13)</f>
+        <v/>
+      </c>
+      <c r="AG13">
+        <f>AD13+AE13</f>
+        <v/>
+      </c>
+      <c r="AH13">
+        <f>Settings!$B$2+AF13</f>
+        <v/>
+      </c>
+      <c r="AI13">
+        <f>AH13-AG13</f>
+        <v/>
+      </c>
+      <c r="AJ13">
+        <f>IF(OR(AND(C13&gt;0,W13=0),AND(E13&gt;0,Y13=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG13&gt;AH13,"ERROR: Rounded balance broken",IF(AI13&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -4357,6 +4721,34 @@
         <f>IF(AB14="FIXED","Close adjusted by SAFE mode",IF(AB14="SAFE","BUY/SELL balance preserved",IF(AB14="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD14">
+        <f>MAX(0,Settings!$B$2*G14/100-AA14)</f>
+        <v/>
+      </c>
+      <c r="AE14">
+        <f>SUM($W$3:W14)</f>
+        <v/>
+      </c>
+      <c r="AF14">
+        <f>SUM($Y$3:Y14)</f>
+        <v/>
+      </c>
+      <c r="AG14">
+        <f>AD14+AE14</f>
+        <v/>
+      </c>
+      <c r="AH14">
+        <f>Settings!$B$2+AF14</f>
+        <v/>
+      </c>
+      <c r="AI14">
+        <f>AH14-AG14</f>
+        <v/>
+      </c>
+      <c r="AJ14">
+        <f>IF(OR(AND(C14&gt;0,W14=0),AND(E14&gt;0,Y14=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG14&gt;AH14,"ERROR: Rounded balance broken",IF(AI14&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -4474,6 +4866,34 @@
         <f>IF(AB15="FIXED","Close adjusted by SAFE mode",IF(AB15="SAFE","BUY/SELL balance preserved",IF(AB15="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD15">
+        <f>MAX(0,Settings!$B$2*G15/100-AA15)</f>
+        <v/>
+      </c>
+      <c r="AE15">
+        <f>SUM($W$3:W15)</f>
+        <v/>
+      </c>
+      <c r="AF15">
+        <f>SUM($Y$3:Y15)</f>
+        <v/>
+      </c>
+      <c r="AG15">
+        <f>AD15+AE15</f>
+        <v/>
+      </c>
+      <c r="AH15">
+        <f>Settings!$B$2+AF15</f>
+        <v/>
+      </c>
+      <c r="AI15">
+        <f>AH15-AG15</f>
+        <v/>
+      </c>
+      <c r="AJ15">
+        <f>IF(OR(AND(C15&gt;0,W15=0),AND(E15&gt;0,Y15=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG15&gt;AH15,"ERROR: Rounded balance broken",IF(AI15&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -4591,6 +5011,34 @@
         <f>IF(AB16="FIXED","Close adjusted by SAFE mode",IF(AB16="SAFE","BUY/SELL balance preserved",IF(AB16="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD16">
+        <f>MAX(0,Settings!$B$2*G16/100-AA16)</f>
+        <v/>
+      </c>
+      <c r="AE16">
+        <f>SUM($W$3:W16)</f>
+        <v/>
+      </c>
+      <c r="AF16">
+        <f>SUM($Y$3:Y16)</f>
+        <v/>
+      </c>
+      <c r="AG16">
+        <f>AD16+AE16</f>
+        <v/>
+      </c>
+      <c r="AH16">
+        <f>Settings!$B$2+AF16</f>
+        <v/>
+      </c>
+      <c r="AI16">
+        <f>AH16-AG16</f>
+        <v/>
+      </c>
+      <c r="AJ16">
+        <f>IF(OR(AND(C16&gt;0,W16=0),AND(E16&gt;0,Y16=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG16&gt;AH16,"ERROR: Rounded balance broken",IF(AI16&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -4708,6 +5156,34 @@
         <f>IF(AB17="FIXED","Close adjusted by SAFE mode",IF(AB17="SAFE","BUY/SELL balance preserved",IF(AB17="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD17">
+        <f>MAX(0,Settings!$B$2*G17/100-AA17)</f>
+        <v/>
+      </c>
+      <c r="AE17">
+        <f>SUM($W$3:W17)</f>
+        <v/>
+      </c>
+      <c r="AF17">
+        <f>SUM($Y$3:Y17)</f>
+        <v/>
+      </c>
+      <c r="AG17">
+        <f>AD17+AE17</f>
+        <v/>
+      </c>
+      <c r="AH17">
+        <f>Settings!$B$2+AF17</f>
+        <v/>
+      </c>
+      <c r="AI17">
+        <f>AH17-AG17</f>
+        <v/>
+      </c>
+      <c r="AJ17">
+        <f>IF(OR(AND(C17&gt;0,W17=0),AND(E17&gt;0,Y17=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG17&gt;AH17,"ERROR: Rounded balance broken",IF(AI17&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -4825,6 +5301,34 @@
         <f>IF(AB18="FIXED","Close adjusted by SAFE mode",IF(AB18="SAFE","BUY/SELL balance preserved",IF(AB18="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD18">
+        <f>MAX(0,Settings!$B$2*G18/100-AA18)</f>
+        <v/>
+      </c>
+      <c r="AE18">
+        <f>SUM($W$3:W18)</f>
+        <v/>
+      </c>
+      <c r="AF18">
+        <f>SUM($Y$3:Y18)</f>
+        <v/>
+      </c>
+      <c r="AG18">
+        <f>AD18+AE18</f>
+        <v/>
+      </c>
+      <c r="AH18">
+        <f>Settings!$B$2+AF18</f>
+        <v/>
+      </c>
+      <c r="AI18">
+        <f>AH18-AG18</f>
+        <v/>
+      </c>
+      <c r="AJ18">
+        <f>IF(OR(AND(C18&gt;0,W18=0),AND(E18&gt;0,Y18=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG18&gt;AH18,"ERROR: Rounded balance broken",IF(AI18&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -4942,6 +5446,34 @@
         <f>IF(AB19="FIXED","Close adjusted by SAFE mode",IF(AB19="SAFE","BUY/SELL balance preserved",IF(AB19="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD19">
+        <f>MAX(0,Settings!$B$2*G19/100-AA19)</f>
+        <v/>
+      </c>
+      <c r="AE19">
+        <f>SUM($W$3:W19)</f>
+        <v/>
+      </c>
+      <c r="AF19">
+        <f>SUM($Y$3:Y19)</f>
+        <v/>
+      </c>
+      <c r="AG19">
+        <f>AD19+AE19</f>
+        <v/>
+      </c>
+      <c r="AH19">
+        <f>Settings!$B$2+AF19</f>
+        <v/>
+      </c>
+      <c r="AI19">
+        <f>AH19-AG19</f>
+        <v/>
+      </c>
+      <c r="AJ19">
+        <f>IF(OR(AND(C19&gt;0,W19=0),AND(E19&gt;0,Y19=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG19&gt;AH19,"ERROR: Rounded balance broken",IF(AI19&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -5059,6 +5591,34 @@
         <f>IF(AB20="FIXED","Close adjusted by SAFE mode",IF(AB20="SAFE","BUY/SELL balance preserved",IF(AB20="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD20">
+        <f>MAX(0,Settings!$B$2*G20/100-AA20)</f>
+        <v/>
+      </c>
+      <c r="AE20">
+        <f>SUM($W$3:W20)</f>
+        <v/>
+      </c>
+      <c r="AF20">
+        <f>SUM($Y$3:Y20)</f>
+        <v/>
+      </c>
+      <c r="AG20">
+        <f>AD20+AE20</f>
+        <v/>
+      </c>
+      <c r="AH20">
+        <f>Settings!$B$2+AF20</f>
+        <v/>
+      </c>
+      <c r="AI20">
+        <f>AH20-AG20</f>
+        <v/>
+      </c>
+      <c r="AJ20">
+        <f>IF(OR(AND(C20&gt;0,W20=0),AND(E20&gt;0,Y20=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG20&gt;AH20,"ERROR: Rounded balance broken",IF(AI20&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -5176,6 +5736,34 @@
         <f>IF(AB21="FIXED","Close adjusted by SAFE mode",IF(AB21="SAFE","BUY/SELL balance preserved",IF(AB21="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD21">
+        <f>MAX(0,Settings!$B$2*G21/100-AA21)</f>
+        <v/>
+      </c>
+      <c r="AE21">
+        <f>SUM($W$3:W21)</f>
+        <v/>
+      </c>
+      <c r="AF21">
+        <f>SUM($Y$3:Y21)</f>
+        <v/>
+      </c>
+      <c r="AG21">
+        <f>AD21+AE21</f>
+        <v/>
+      </c>
+      <c r="AH21">
+        <f>Settings!$B$2+AF21</f>
+        <v/>
+      </c>
+      <c r="AI21">
+        <f>AH21-AG21</f>
+        <v/>
+      </c>
+      <c r="AJ21">
+        <f>IF(OR(AND(C21&gt;0,W21=0),AND(E21&gt;0,Y21=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG21&gt;AH21,"ERROR: Rounded balance broken",IF(AI21&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -5293,6 +5881,34 @@
         <f>IF(AB22="FIXED","Close adjusted by SAFE mode",IF(AB22="SAFE","BUY/SELL balance preserved",IF(AB22="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD22">
+        <f>MAX(0,Settings!$B$2*G22/100-AA22)</f>
+        <v/>
+      </c>
+      <c r="AE22">
+        <f>SUM($W$3:W22)</f>
+        <v/>
+      </c>
+      <c r="AF22">
+        <f>SUM($Y$3:Y22)</f>
+        <v/>
+      </c>
+      <c r="AG22">
+        <f>AD22+AE22</f>
+        <v/>
+      </c>
+      <c r="AH22">
+        <f>Settings!$B$2+AF22</f>
+        <v/>
+      </c>
+      <c r="AI22">
+        <f>AH22-AG22</f>
+        <v/>
+      </c>
+      <c r="AJ22">
+        <f>IF(OR(AND(C22&gt;0,W22=0),AND(E22&gt;0,Y22=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG22&gt;AH22,"ERROR: Rounded balance broken",IF(AI22&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -5410,6 +6026,34 @@
         <f>IF(AB23="FIXED","Close adjusted by SAFE mode",IF(AB23="SAFE","BUY/SELL balance preserved",IF(AB23="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD23">
+        <f>MAX(0,Settings!$B$2*G23/100-AA23)</f>
+        <v/>
+      </c>
+      <c r="AE23">
+        <f>SUM($W$3:W23)</f>
+        <v/>
+      </c>
+      <c r="AF23">
+        <f>SUM($Y$3:Y23)</f>
+        <v/>
+      </c>
+      <c r="AG23">
+        <f>AD23+AE23</f>
+        <v/>
+      </c>
+      <c r="AH23">
+        <f>Settings!$B$2+AF23</f>
+        <v/>
+      </c>
+      <c r="AI23">
+        <f>AH23-AG23</f>
+        <v/>
+      </c>
+      <c r="AJ23">
+        <f>IF(OR(AND(C23&gt;0,W23=0),AND(E23&gt;0,Y23=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG23&gt;AH23,"ERROR: Rounded balance broken",IF(AI23&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -5527,6 +6171,34 @@
         <f>IF(AB24="FIXED","Close adjusted by SAFE mode",IF(AB24="SAFE","BUY/SELL balance preserved",IF(AB24="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD24">
+        <f>MAX(0,Settings!$B$2*G24/100-AA24)</f>
+        <v/>
+      </c>
+      <c r="AE24">
+        <f>SUM($W$3:W24)</f>
+        <v/>
+      </c>
+      <c r="AF24">
+        <f>SUM($Y$3:Y24)</f>
+        <v/>
+      </c>
+      <c r="AG24">
+        <f>AD24+AE24</f>
+        <v/>
+      </c>
+      <c r="AH24">
+        <f>Settings!$B$2+AF24</f>
+        <v/>
+      </c>
+      <c r="AI24">
+        <f>AH24-AG24</f>
+        <v/>
+      </c>
+      <c r="AJ24">
+        <f>IF(OR(AND(C24&gt;0,W24=0),AND(E24&gt;0,Y24=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG24&gt;AH24,"ERROR: Rounded balance broken",IF(AI24&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -5644,6 +6316,34 @@
         <f>IF(AB25="FIXED","Close adjusted by SAFE mode",IF(AB25="SAFE","BUY/SELL balance preserved",IF(AB25="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD25">
+        <f>MAX(0,Settings!$B$2*G25/100-AA25)</f>
+        <v/>
+      </c>
+      <c r="AE25">
+        <f>SUM($W$3:W25)</f>
+        <v/>
+      </c>
+      <c r="AF25">
+        <f>SUM($Y$3:Y25)</f>
+        <v/>
+      </c>
+      <c r="AG25">
+        <f>AD25+AE25</f>
+        <v/>
+      </c>
+      <c r="AH25">
+        <f>Settings!$B$2+AF25</f>
+        <v/>
+      </c>
+      <c r="AI25">
+        <f>AH25-AG25</f>
+        <v/>
+      </c>
+      <c r="AJ25">
+        <f>IF(OR(AND(C25&gt;0,W25=0),AND(E25&gt;0,Y25=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG25&gt;AH25,"ERROR: Rounded balance broken",IF(AI25&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -5761,6 +6461,34 @@
         <f>IF(AB26="FIXED","Close adjusted by SAFE mode",IF(AB26="SAFE","BUY/SELL balance preserved",IF(AB26="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD26">
+        <f>MAX(0,Settings!$B$2*G26/100-AA26)</f>
+        <v/>
+      </c>
+      <c r="AE26">
+        <f>SUM($W$3:W26)</f>
+        <v/>
+      </c>
+      <c r="AF26">
+        <f>SUM($Y$3:Y26)</f>
+        <v/>
+      </c>
+      <c r="AG26">
+        <f>AD26+AE26</f>
+        <v/>
+      </c>
+      <c r="AH26">
+        <f>Settings!$B$2+AF26</f>
+        <v/>
+      </c>
+      <c r="AI26">
+        <f>AH26-AG26</f>
+        <v/>
+      </c>
+      <c r="AJ26">
+        <f>IF(OR(AND(C26&gt;0,W26=0),AND(E26&gt;0,Y26=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG26&gt;AH26,"ERROR: Rounded balance broken",IF(AI26&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -5878,6 +6606,34 @@
         <f>IF(AB27="FIXED","Close adjusted by SAFE mode",IF(AB27="SAFE","BUY/SELL balance preserved",IF(AB27="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD27">
+        <f>MAX(0,Settings!$B$2*G27/100-AA27)</f>
+        <v/>
+      </c>
+      <c r="AE27">
+        <f>SUM($W$3:W27)</f>
+        <v/>
+      </c>
+      <c r="AF27">
+        <f>SUM($Y$3:Y27)</f>
+        <v/>
+      </c>
+      <c r="AG27">
+        <f>AD27+AE27</f>
+        <v/>
+      </c>
+      <c r="AH27">
+        <f>Settings!$B$2+AF27</f>
+        <v/>
+      </c>
+      <c r="AI27">
+        <f>AH27-AG27</f>
+        <v/>
+      </c>
+      <c r="AJ27">
+        <f>IF(OR(AND(C27&gt;0,W27=0),AND(E27&gt;0,Y27=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG27&gt;AH27,"ERROR: Rounded balance broken",IF(AI27&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -5995,6 +6751,34 @@
         <f>IF(AB28="FIXED","Close adjusted by SAFE mode",IF(AB28="SAFE","BUY/SELL balance preserved",IF(AB28="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD28">
+        <f>MAX(0,Settings!$B$2*G28/100-AA28)</f>
+        <v/>
+      </c>
+      <c r="AE28">
+        <f>SUM($W$3:W28)</f>
+        <v/>
+      </c>
+      <c r="AF28">
+        <f>SUM($Y$3:Y28)</f>
+        <v/>
+      </c>
+      <c r="AG28">
+        <f>AD28+AE28</f>
+        <v/>
+      </c>
+      <c r="AH28">
+        <f>Settings!$B$2+AF28</f>
+        <v/>
+      </c>
+      <c r="AI28">
+        <f>AH28-AG28</f>
+        <v/>
+      </c>
+      <c r="AJ28">
+        <f>IF(OR(AND(C28&gt;0,W28=0),AND(E28&gt;0,Y28=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG28&gt;AH28,"ERROR: Rounded balance broken",IF(AI28&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -6112,6 +6896,34 @@
         <f>IF(AB29="FIXED","Close adjusted by SAFE mode",IF(AB29="SAFE","BUY/SELL balance preserved",IF(AB29="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD29">
+        <f>MAX(0,Settings!$B$2*G29/100-AA29)</f>
+        <v/>
+      </c>
+      <c r="AE29">
+        <f>SUM($W$3:W29)</f>
+        <v/>
+      </c>
+      <c r="AF29">
+        <f>SUM($Y$3:Y29)</f>
+        <v/>
+      </c>
+      <c r="AG29">
+        <f>AD29+AE29</f>
+        <v/>
+      </c>
+      <c r="AH29">
+        <f>Settings!$B$2+AF29</f>
+        <v/>
+      </c>
+      <c r="AI29">
+        <f>AH29-AG29</f>
+        <v/>
+      </c>
+      <c r="AJ29">
+        <f>IF(OR(AND(C29&gt;0,W29=0),AND(E29&gt;0,Y29=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG29&gt;AH29,"ERROR: Rounded balance broken",IF(AI29&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -6229,6 +7041,34 @@
         <f>IF(AB30="FIXED","Close adjusted by SAFE mode",IF(AB30="SAFE","BUY/SELL balance preserved",IF(AB30="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD30">
+        <f>MAX(0,Settings!$B$2*G30/100-AA30)</f>
+        <v/>
+      </c>
+      <c r="AE30">
+        <f>SUM($W$3:W30)</f>
+        <v/>
+      </c>
+      <c r="AF30">
+        <f>SUM($Y$3:Y30)</f>
+        <v/>
+      </c>
+      <c r="AG30">
+        <f>AD30+AE30</f>
+        <v/>
+      </c>
+      <c r="AH30">
+        <f>Settings!$B$2+AF30</f>
+        <v/>
+      </c>
+      <c r="AI30">
+        <f>AH30-AG30</f>
+        <v/>
+      </c>
+      <c r="AJ30">
+        <f>IF(OR(AND(C30&gt;0,W30=0),AND(E30&gt;0,Y30=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG30&gt;AH30,"ERROR: Rounded balance broken",IF(AI30&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -6346,6 +7186,34 @@
         <f>IF(AB31="FIXED","Close adjusted by SAFE mode",IF(AB31="SAFE","BUY/SELL balance preserved",IF(AB31="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD31">
+        <f>MAX(0,Settings!$B$2*G31/100-AA31)</f>
+        <v/>
+      </c>
+      <c r="AE31">
+        <f>SUM($W$3:W31)</f>
+        <v/>
+      </c>
+      <c r="AF31">
+        <f>SUM($Y$3:Y31)</f>
+        <v/>
+      </c>
+      <c r="AG31">
+        <f>AD31+AE31</f>
+        <v/>
+      </c>
+      <c r="AH31">
+        <f>Settings!$B$2+AF31</f>
+        <v/>
+      </c>
+      <c r="AI31">
+        <f>AH31-AG31</f>
+        <v/>
+      </c>
+      <c r="AJ31">
+        <f>IF(OR(AND(C31&gt;0,W31=0),AND(E31&gt;0,Y31=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG31&gt;AH31,"ERROR: Rounded balance broken",IF(AI31&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -6463,6 +7331,34 @@
         <f>IF(AB32="FIXED","Close adjusted by SAFE mode",IF(AB32="SAFE","BUY/SELL balance preserved",IF(AB32="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD32">
+        <f>MAX(0,Settings!$B$2*G32/100-AA32)</f>
+        <v/>
+      </c>
+      <c r="AE32">
+        <f>SUM($W$3:W32)</f>
+        <v/>
+      </c>
+      <c r="AF32">
+        <f>SUM($Y$3:Y32)</f>
+        <v/>
+      </c>
+      <c r="AG32">
+        <f>AD32+AE32</f>
+        <v/>
+      </c>
+      <c r="AH32">
+        <f>Settings!$B$2+AF32</f>
+        <v/>
+      </c>
+      <c r="AI32">
+        <f>AH32-AG32</f>
+        <v/>
+      </c>
+      <c r="AJ32">
+        <f>IF(OR(AND(C32&gt;0,W32=0),AND(E32&gt;0,Y32=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG32&gt;AH32,"ERROR: Rounded balance broken",IF(AI32&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -6580,6 +7476,34 @@
         <f>IF(AB33="FIXED","Close adjusted by SAFE mode",IF(AB33="SAFE","BUY/SELL balance preserved",IF(AB33="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD33">
+        <f>MAX(0,Settings!$B$2*G33/100-AA33)</f>
+        <v/>
+      </c>
+      <c r="AE33">
+        <f>SUM($W$3:W33)</f>
+        <v/>
+      </c>
+      <c r="AF33">
+        <f>SUM($Y$3:Y33)</f>
+        <v/>
+      </c>
+      <c r="AG33">
+        <f>AD33+AE33</f>
+        <v/>
+      </c>
+      <c r="AH33">
+        <f>Settings!$B$2+AF33</f>
+        <v/>
+      </c>
+      <c r="AI33">
+        <f>AH33-AG33</f>
+        <v/>
+      </c>
+      <c r="AJ33">
+        <f>IF(OR(AND(C33&gt;0,W33=0),AND(E33&gt;0,Y33=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG33&gt;AH33,"ERROR: Rounded balance broken",IF(AI33&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -6697,6 +7621,34 @@
         <f>IF(AB34="FIXED","Close adjusted by SAFE mode",IF(AB34="SAFE","BUY/SELL balance preserved",IF(AB34="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD34">
+        <f>MAX(0,Settings!$B$2*G34/100-AA34)</f>
+        <v/>
+      </c>
+      <c r="AE34">
+        <f>SUM($W$3:W34)</f>
+        <v/>
+      </c>
+      <c r="AF34">
+        <f>SUM($Y$3:Y34)</f>
+        <v/>
+      </c>
+      <c r="AG34">
+        <f>AD34+AE34</f>
+        <v/>
+      </c>
+      <c r="AH34">
+        <f>Settings!$B$2+AF34</f>
+        <v/>
+      </c>
+      <c r="AI34">
+        <f>AH34-AG34</f>
+        <v/>
+      </c>
+      <c r="AJ34">
+        <f>IF(OR(AND(C34&gt;0,W34=0),AND(E34&gt;0,Y34=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG34&gt;AH34,"ERROR: Rounded balance broken",IF(AI34&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -6814,6 +7766,34 @@
         <f>IF(AB35="FIXED","Close adjusted by SAFE mode",IF(AB35="SAFE","BUY/SELL balance preserved",IF(AB35="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD35">
+        <f>MAX(0,Settings!$B$2*G35/100-AA35)</f>
+        <v/>
+      </c>
+      <c r="AE35">
+        <f>SUM($W$3:W35)</f>
+        <v/>
+      </c>
+      <c r="AF35">
+        <f>SUM($Y$3:Y35)</f>
+        <v/>
+      </c>
+      <c r="AG35">
+        <f>AD35+AE35</f>
+        <v/>
+      </c>
+      <c r="AH35">
+        <f>Settings!$B$2+AF35</f>
+        <v/>
+      </c>
+      <c r="AI35">
+        <f>AH35-AG35</f>
+        <v/>
+      </c>
+      <c r="AJ35">
+        <f>IF(OR(AND(C35&gt;0,W35=0),AND(E35&gt;0,Y35=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG35&gt;AH35,"ERROR: Rounded balance broken",IF(AI35&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -6931,6 +7911,34 @@
         <f>IF(AB36="FIXED","Close adjusted by SAFE mode",IF(AB36="SAFE","BUY/SELL balance preserved",IF(AB36="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD36">
+        <f>MAX(0,Settings!$B$2*G36/100-AA36)</f>
+        <v/>
+      </c>
+      <c r="AE36">
+        <f>SUM($W$3:W36)</f>
+        <v/>
+      </c>
+      <c r="AF36">
+        <f>SUM($Y$3:Y36)</f>
+        <v/>
+      </c>
+      <c r="AG36">
+        <f>AD36+AE36</f>
+        <v/>
+      </c>
+      <c r="AH36">
+        <f>Settings!$B$2+AF36</f>
+        <v/>
+      </c>
+      <c r="AI36">
+        <f>AH36-AG36</f>
+        <v/>
+      </c>
+      <c r="AJ36">
+        <f>IF(OR(AND(C36&gt;0,W36=0),AND(E36&gt;0,Y36=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG36&gt;AH36,"ERROR: Rounded balance broken",IF(AI36&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -7048,6 +8056,34 @@
         <f>IF(AB37="FIXED","Close adjusted by SAFE mode",IF(AB37="SAFE","BUY/SELL balance preserved",IF(AB37="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD37">
+        <f>MAX(0,Settings!$B$2*G37/100-AA37)</f>
+        <v/>
+      </c>
+      <c r="AE37">
+        <f>SUM($W$3:W37)</f>
+        <v/>
+      </c>
+      <c r="AF37">
+        <f>SUM($Y$3:Y37)</f>
+        <v/>
+      </c>
+      <c r="AG37">
+        <f>AD37+AE37</f>
+        <v/>
+      </c>
+      <c r="AH37">
+        <f>Settings!$B$2+AF37</f>
+        <v/>
+      </c>
+      <c r="AI37">
+        <f>AH37-AG37</f>
+        <v/>
+      </c>
+      <c r="AJ37">
+        <f>IF(OR(AND(C37&gt;0,W37=0),AND(E37&gt;0,Y37=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG37&gt;AH37,"ERROR: Rounded balance broken",IF(AI37&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -7165,6 +8201,34 @@
         <f>IF(AB38="FIXED","Close adjusted by SAFE mode",IF(AB38="SAFE","BUY/SELL balance preserved",IF(AB38="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD38">
+        <f>MAX(0,Settings!$B$2*G38/100-AA38)</f>
+        <v/>
+      </c>
+      <c r="AE38">
+        <f>SUM($W$3:W38)</f>
+        <v/>
+      </c>
+      <c r="AF38">
+        <f>SUM($Y$3:Y38)</f>
+        <v/>
+      </c>
+      <c r="AG38">
+        <f>AD38+AE38</f>
+        <v/>
+      </c>
+      <c r="AH38">
+        <f>Settings!$B$2+AF38</f>
+        <v/>
+      </c>
+      <c r="AI38">
+        <f>AH38-AG38</f>
+        <v/>
+      </c>
+      <c r="AJ38">
+        <f>IF(OR(AND(C38&gt;0,W38=0),AND(E38&gt;0,Y38=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG38&gt;AH38,"ERROR: Rounded balance broken",IF(AI38&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -7282,6 +8346,34 @@
         <f>IF(AB39="FIXED","Close adjusted by SAFE mode",IF(AB39="SAFE","BUY/SELL balance preserved",IF(AB39="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD39">
+        <f>MAX(0,Settings!$B$2*G39/100-AA39)</f>
+        <v/>
+      </c>
+      <c r="AE39">
+        <f>SUM($W$3:W39)</f>
+        <v/>
+      </c>
+      <c r="AF39">
+        <f>SUM($Y$3:Y39)</f>
+        <v/>
+      </c>
+      <c r="AG39">
+        <f>AD39+AE39</f>
+        <v/>
+      </c>
+      <c r="AH39">
+        <f>Settings!$B$2+AF39</f>
+        <v/>
+      </c>
+      <c r="AI39">
+        <f>AH39-AG39</f>
+        <v/>
+      </c>
+      <c r="AJ39">
+        <f>IF(OR(AND(C39&gt;0,W39=0),AND(E39&gt;0,Y39=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG39&gt;AH39,"ERROR: Rounded balance broken",IF(AI39&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -7399,6 +8491,34 @@
         <f>IF(AB40="FIXED","Close adjusted by SAFE mode",IF(AB40="SAFE","BUY/SELL balance preserved",IF(AB40="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD40">
+        <f>MAX(0,Settings!$B$2*G40/100-AA40)</f>
+        <v/>
+      </c>
+      <c r="AE40">
+        <f>SUM($W$3:W40)</f>
+        <v/>
+      </c>
+      <c r="AF40">
+        <f>SUM($Y$3:Y40)</f>
+        <v/>
+      </c>
+      <c r="AG40">
+        <f>AD40+AE40</f>
+        <v/>
+      </c>
+      <c r="AH40">
+        <f>Settings!$B$2+AF40</f>
+        <v/>
+      </c>
+      <c r="AI40">
+        <f>AH40-AG40</f>
+        <v/>
+      </c>
+      <c r="AJ40">
+        <f>IF(OR(AND(C40&gt;0,W40=0),AND(E40&gt;0,Y40=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG40&gt;AH40,"ERROR: Rounded balance broken",IF(AI40&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -7514,6 +8634,34 @@
       </c>
       <c r="AC41">
         <f>IF(AB41="FIXED","Close adjusted by SAFE mode",IF(AB41="SAFE","BUY/SELL balance preserved",IF(AB41="WARNING","Near protection boundary","Protection broken")))</f>
+        <v/>
+      </c>
+      <c r="AD41">
+        <f>MAX(0,Settings!$B$2*G41/100-AA41)</f>
+        <v/>
+      </c>
+      <c r="AE41">
+        <f>SUM($W$3:W41)</f>
+        <v/>
+      </c>
+      <c r="AF41">
+        <f>SUM($Y$3:Y41)</f>
+        <v/>
+      </c>
+      <c r="AG41">
+        <f>AD41+AE41</f>
+        <v/>
+      </c>
+      <c r="AH41">
+        <f>Settings!$B$2+AF41</f>
+        <v/>
+      </c>
+      <c r="AI41">
+        <f>AH41-AG41</f>
+        <v/>
+      </c>
+      <c r="AJ41">
+        <f>IF(OR(AND(C41&gt;0,W41=0),AND(E41&gt;0,Y41=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG41&gt;AH41,"ERROR: Rounded balance broken",IF(AI41&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -7542,7 +8690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC41"/>
+  <dimension ref="A1:AJ41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7691,6 +8839,41 @@
           <t>Rounding Comment</t>
         </is>
       </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>Rounded Start After Lot</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Rounded Sum Big Lot</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Rounded Sum Small Lot</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Rounded Total Main Lot</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Rounded Total Opposite Lot</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>Rounded Skew Lot</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>Rounded Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -7787,6 +8970,27 @@
         <f>IF(AB2="FIXED","Close adjusted by SAFE mode",IF(AB2="SAFE","BUY/SELL balance preserved",IF(AB2="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -7903,6 +9107,34 @@
         <f>IF(AB3="FIXED","Close adjusted by SAFE mode",IF(AB3="SAFE","BUY/SELL balance preserved",IF(AB3="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD3">
+        <f>MAX(0,Settings!$B$2*G3/100-AA3)</f>
+        <v/>
+      </c>
+      <c r="AE3">
+        <f>SUM($W$3:W3)</f>
+        <v/>
+      </c>
+      <c r="AF3">
+        <f>SUM($Y$3:Y3)</f>
+        <v/>
+      </c>
+      <c r="AG3">
+        <f>AD3+AE3</f>
+        <v/>
+      </c>
+      <c r="AH3">
+        <f>Settings!$B$2+AF3</f>
+        <v/>
+      </c>
+      <c r="AI3">
+        <f>AH3-AG3</f>
+        <v/>
+      </c>
+      <c r="AJ3">
+        <f>IF(OR(AND(C3&gt;0,W3=0),AND(E3&gt;0,Y3=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG3&gt;AH3,"ERROR: Rounded balance broken",IF(AI3&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -8020,6 +9252,34 @@
         <f>IF(AB4="FIXED","Close adjusted by SAFE mode",IF(AB4="SAFE","BUY/SELL balance preserved",IF(AB4="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD4">
+        <f>MAX(0,Settings!$B$2*G4/100-AA4)</f>
+        <v/>
+      </c>
+      <c r="AE4">
+        <f>SUM($W$3:W4)</f>
+        <v/>
+      </c>
+      <c r="AF4">
+        <f>SUM($Y$3:Y4)</f>
+        <v/>
+      </c>
+      <c r="AG4">
+        <f>AD4+AE4</f>
+        <v/>
+      </c>
+      <c r="AH4">
+        <f>Settings!$B$2+AF4</f>
+        <v/>
+      </c>
+      <c r="AI4">
+        <f>AH4-AG4</f>
+        <v/>
+      </c>
+      <c r="AJ4">
+        <f>IF(OR(AND(C4&gt;0,W4=0),AND(E4&gt;0,Y4=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG4&gt;AH4,"ERROR: Rounded balance broken",IF(AI4&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -8137,6 +9397,34 @@
         <f>IF(AB5="FIXED","Close adjusted by SAFE mode",IF(AB5="SAFE","BUY/SELL balance preserved",IF(AB5="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD5">
+        <f>MAX(0,Settings!$B$2*G5/100-AA5)</f>
+        <v/>
+      </c>
+      <c r="AE5">
+        <f>SUM($W$3:W5)</f>
+        <v/>
+      </c>
+      <c r="AF5">
+        <f>SUM($Y$3:Y5)</f>
+        <v/>
+      </c>
+      <c r="AG5">
+        <f>AD5+AE5</f>
+        <v/>
+      </c>
+      <c r="AH5">
+        <f>Settings!$B$2+AF5</f>
+        <v/>
+      </c>
+      <c r="AI5">
+        <f>AH5-AG5</f>
+        <v/>
+      </c>
+      <c r="AJ5">
+        <f>IF(OR(AND(C5&gt;0,W5=0),AND(E5&gt;0,Y5=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG5&gt;AH5,"ERROR: Rounded balance broken",IF(AI5&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -8254,6 +9542,34 @@
         <f>IF(AB6="FIXED","Close adjusted by SAFE mode",IF(AB6="SAFE","BUY/SELL balance preserved",IF(AB6="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD6">
+        <f>MAX(0,Settings!$B$2*G6/100-AA6)</f>
+        <v/>
+      </c>
+      <c r="AE6">
+        <f>SUM($W$3:W6)</f>
+        <v/>
+      </c>
+      <c r="AF6">
+        <f>SUM($Y$3:Y6)</f>
+        <v/>
+      </c>
+      <c r="AG6">
+        <f>AD6+AE6</f>
+        <v/>
+      </c>
+      <c r="AH6">
+        <f>Settings!$B$2+AF6</f>
+        <v/>
+      </c>
+      <c r="AI6">
+        <f>AH6-AG6</f>
+        <v/>
+      </c>
+      <c r="AJ6">
+        <f>IF(OR(AND(C6&gt;0,W6=0),AND(E6&gt;0,Y6=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG6&gt;AH6,"ERROR: Rounded balance broken",IF(AI6&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -8371,6 +9687,34 @@
         <f>IF(AB7="FIXED","Close adjusted by SAFE mode",IF(AB7="SAFE","BUY/SELL balance preserved",IF(AB7="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD7">
+        <f>MAX(0,Settings!$B$2*G7/100-AA7)</f>
+        <v/>
+      </c>
+      <c r="AE7">
+        <f>SUM($W$3:W7)</f>
+        <v/>
+      </c>
+      <c r="AF7">
+        <f>SUM($Y$3:Y7)</f>
+        <v/>
+      </c>
+      <c r="AG7">
+        <f>AD7+AE7</f>
+        <v/>
+      </c>
+      <c r="AH7">
+        <f>Settings!$B$2+AF7</f>
+        <v/>
+      </c>
+      <c r="AI7">
+        <f>AH7-AG7</f>
+        <v/>
+      </c>
+      <c r="AJ7">
+        <f>IF(OR(AND(C7&gt;0,W7=0),AND(E7&gt;0,Y7=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG7&gt;AH7,"ERROR: Rounded balance broken",IF(AI7&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -8488,6 +9832,34 @@
         <f>IF(AB8="FIXED","Close adjusted by SAFE mode",IF(AB8="SAFE","BUY/SELL balance preserved",IF(AB8="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD8">
+        <f>MAX(0,Settings!$B$2*G8/100-AA8)</f>
+        <v/>
+      </c>
+      <c r="AE8">
+        <f>SUM($W$3:W8)</f>
+        <v/>
+      </c>
+      <c r="AF8">
+        <f>SUM($Y$3:Y8)</f>
+        <v/>
+      </c>
+      <c r="AG8">
+        <f>AD8+AE8</f>
+        <v/>
+      </c>
+      <c r="AH8">
+        <f>Settings!$B$2+AF8</f>
+        <v/>
+      </c>
+      <c r="AI8">
+        <f>AH8-AG8</f>
+        <v/>
+      </c>
+      <c r="AJ8">
+        <f>IF(OR(AND(C8&gt;0,W8=0),AND(E8&gt;0,Y8=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG8&gt;AH8,"ERROR: Rounded balance broken",IF(AI8&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -8605,6 +9977,34 @@
         <f>IF(AB9="FIXED","Close adjusted by SAFE mode",IF(AB9="SAFE","BUY/SELL balance preserved",IF(AB9="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD9">
+        <f>MAX(0,Settings!$B$2*G9/100-AA9)</f>
+        <v/>
+      </c>
+      <c r="AE9">
+        <f>SUM($W$3:W9)</f>
+        <v/>
+      </c>
+      <c r="AF9">
+        <f>SUM($Y$3:Y9)</f>
+        <v/>
+      </c>
+      <c r="AG9">
+        <f>AD9+AE9</f>
+        <v/>
+      </c>
+      <c r="AH9">
+        <f>Settings!$B$2+AF9</f>
+        <v/>
+      </c>
+      <c r="AI9">
+        <f>AH9-AG9</f>
+        <v/>
+      </c>
+      <c r="AJ9">
+        <f>IF(OR(AND(C9&gt;0,W9=0),AND(E9&gt;0,Y9=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG9&gt;AH9,"ERROR: Rounded balance broken",IF(AI9&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -8722,6 +10122,34 @@
         <f>IF(AB10="FIXED","Close adjusted by SAFE mode",IF(AB10="SAFE","BUY/SELL balance preserved",IF(AB10="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD10">
+        <f>MAX(0,Settings!$B$2*G10/100-AA10)</f>
+        <v/>
+      </c>
+      <c r="AE10">
+        <f>SUM($W$3:W10)</f>
+        <v/>
+      </c>
+      <c r="AF10">
+        <f>SUM($Y$3:Y10)</f>
+        <v/>
+      </c>
+      <c r="AG10">
+        <f>AD10+AE10</f>
+        <v/>
+      </c>
+      <c r="AH10">
+        <f>Settings!$B$2+AF10</f>
+        <v/>
+      </c>
+      <c r="AI10">
+        <f>AH10-AG10</f>
+        <v/>
+      </c>
+      <c r="AJ10">
+        <f>IF(OR(AND(C10&gt;0,W10=0),AND(E10&gt;0,Y10=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG10&gt;AH10,"ERROR: Rounded balance broken",IF(AI10&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -8839,6 +10267,34 @@
         <f>IF(AB11="FIXED","Close adjusted by SAFE mode",IF(AB11="SAFE","BUY/SELL balance preserved",IF(AB11="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD11">
+        <f>MAX(0,Settings!$B$2*G11/100-AA11)</f>
+        <v/>
+      </c>
+      <c r="AE11">
+        <f>SUM($W$3:W11)</f>
+        <v/>
+      </c>
+      <c r="AF11">
+        <f>SUM($Y$3:Y11)</f>
+        <v/>
+      </c>
+      <c r="AG11">
+        <f>AD11+AE11</f>
+        <v/>
+      </c>
+      <c r="AH11">
+        <f>Settings!$B$2+AF11</f>
+        <v/>
+      </c>
+      <c r="AI11">
+        <f>AH11-AG11</f>
+        <v/>
+      </c>
+      <c r="AJ11">
+        <f>IF(OR(AND(C11&gt;0,W11=0),AND(E11&gt;0,Y11=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG11&gt;AH11,"ERROR: Rounded balance broken",IF(AI11&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -8956,6 +10412,34 @@
         <f>IF(AB12="FIXED","Close adjusted by SAFE mode",IF(AB12="SAFE","BUY/SELL balance preserved",IF(AB12="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD12">
+        <f>MAX(0,Settings!$B$2*G12/100-AA12)</f>
+        <v/>
+      </c>
+      <c r="AE12">
+        <f>SUM($W$3:W12)</f>
+        <v/>
+      </c>
+      <c r="AF12">
+        <f>SUM($Y$3:Y12)</f>
+        <v/>
+      </c>
+      <c r="AG12">
+        <f>AD12+AE12</f>
+        <v/>
+      </c>
+      <c r="AH12">
+        <f>Settings!$B$2+AF12</f>
+        <v/>
+      </c>
+      <c r="AI12">
+        <f>AH12-AG12</f>
+        <v/>
+      </c>
+      <c r="AJ12">
+        <f>IF(OR(AND(C12&gt;0,W12=0),AND(E12&gt;0,Y12=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG12&gt;AH12,"ERROR: Rounded balance broken",IF(AI12&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -9073,6 +10557,34 @@
         <f>IF(AB13="FIXED","Close adjusted by SAFE mode",IF(AB13="SAFE","BUY/SELL balance preserved",IF(AB13="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD13">
+        <f>MAX(0,Settings!$B$2*G13/100-AA13)</f>
+        <v/>
+      </c>
+      <c r="AE13">
+        <f>SUM($W$3:W13)</f>
+        <v/>
+      </c>
+      <c r="AF13">
+        <f>SUM($Y$3:Y13)</f>
+        <v/>
+      </c>
+      <c r="AG13">
+        <f>AD13+AE13</f>
+        <v/>
+      </c>
+      <c r="AH13">
+        <f>Settings!$B$2+AF13</f>
+        <v/>
+      </c>
+      <c r="AI13">
+        <f>AH13-AG13</f>
+        <v/>
+      </c>
+      <c r="AJ13">
+        <f>IF(OR(AND(C13&gt;0,W13=0),AND(E13&gt;0,Y13=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG13&gt;AH13,"ERROR: Rounded balance broken",IF(AI13&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -9190,6 +10702,34 @@
         <f>IF(AB14="FIXED","Close adjusted by SAFE mode",IF(AB14="SAFE","BUY/SELL balance preserved",IF(AB14="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD14">
+        <f>MAX(0,Settings!$B$2*G14/100-AA14)</f>
+        <v/>
+      </c>
+      <c r="AE14">
+        <f>SUM($W$3:W14)</f>
+        <v/>
+      </c>
+      <c r="AF14">
+        <f>SUM($Y$3:Y14)</f>
+        <v/>
+      </c>
+      <c r="AG14">
+        <f>AD14+AE14</f>
+        <v/>
+      </c>
+      <c r="AH14">
+        <f>Settings!$B$2+AF14</f>
+        <v/>
+      </c>
+      <c r="AI14">
+        <f>AH14-AG14</f>
+        <v/>
+      </c>
+      <c r="AJ14">
+        <f>IF(OR(AND(C14&gt;0,W14=0),AND(E14&gt;0,Y14=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG14&gt;AH14,"ERROR: Rounded balance broken",IF(AI14&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -9307,6 +10847,34 @@
         <f>IF(AB15="FIXED","Close adjusted by SAFE mode",IF(AB15="SAFE","BUY/SELL balance preserved",IF(AB15="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD15">
+        <f>MAX(0,Settings!$B$2*G15/100-AA15)</f>
+        <v/>
+      </c>
+      <c r="AE15">
+        <f>SUM($W$3:W15)</f>
+        <v/>
+      </c>
+      <c r="AF15">
+        <f>SUM($Y$3:Y15)</f>
+        <v/>
+      </c>
+      <c r="AG15">
+        <f>AD15+AE15</f>
+        <v/>
+      </c>
+      <c r="AH15">
+        <f>Settings!$B$2+AF15</f>
+        <v/>
+      </c>
+      <c r="AI15">
+        <f>AH15-AG15</f>
+        <v/>
+      </c>
+      <c r="AJ15">
+        <f>IF(OR(AND(C15&gt;0,W15=0),AND(E15&gt;0,Y15=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG15&gt;AH15,"ERROR: Rounded balance broken",IF(AI15&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -9424,6 +10992,34 @@
         <f>IF(AB16="FIXED","Close adjusted by SAFE mode",IF(AB16="SAFE","BUY/SELL balance preserved",IF(AB16="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD16">
+        <f>MAX(0,Settings!$B$2*G16/100-AA16)</f>
+        <v/>
+      </c>
+      <c r="AE16">
+        <f>SUM($W$3:W16)</f>
+        <v/>
+      </c>
+      <c r="AF16">
+        <f>SUM($Y$3:Y16)</f>
+        <v/>
+      </c>
+      <c r="AG16">
+        <f>AD16+AE16</f>
+        <v/>
+      </c>
+      <c r="AH16">
+        <f>Settings!$B$2+AF16</f>
+        <v/>
+      </c>
+      <c r="AI16">
+        <f>AH16-AG16</f>
+        <v/>
+      </c>
+      <c r="AJ16">
+        <f>IF(OR(AND(C16&gt;0,W16=0),AND(E16&gt;0,Y16=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG16&gt;AH16,"ERROR: Rounded balance broken",IF(AI16&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -9541,6 +11137,34 @@
         <f>IF(AB17="FIXED","Close adjusted by SAFE mode",IF(AB17="SAFE","BUY/SELL balance preserved",IF(AB17="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD17">
+        <f>MAX(0,Settings!$B$2*G17/100-AA17)</f>
+        <v/>
+      </c>
+      <c r="AE17">
+        <f>SUM($W$3:W17)</f>
+        <v/>
+      </c>
+      <c r="AF17">
+        <f>SUM($Y$3:Y17)</f>
+        <v/>
+      </c>
+      <c r="AG17">
+        <f>AD17+AE17</f>
+        <v/>
+      </c>
+      <c r="AH17">
+        <f>Settings!$B$2+AF17</f>
+        <v/>
+      </c>
+      <c r="AI17">
+        <f>AH17-AG17</f>
+        <v/>
+      </c>
+      <c r="AJ17">
+        <f>IF(OR(AND(C17&gt;0,W17=0),AND(E17&gt;0,Y17=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG17&gt;AH17,"ERROR: Rounded balance broken",IF(AI17&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -9658,6 +11282,34 @@
         <f>IF(AB18="FIXED","Close adjusted by SAFE mode",IF(AB18="SAFE","BUY/SELL balance preserved",IF(AB18="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD18">
+        <f>MAX(0,Settings!$B$2*G18/100-AA18)</f>
+        <v/>
+      </c>
+      <c r="AE18">
+        <f>SUM($W$3:W18)</f>
+        <v/>
+      </c>
+      <c r="AF18">
+        <f>SUM($Y$3:Y18)</f>
+        <v/>
+      </c>
+      <c r="AG18">
+        <f>AD18+AE18</f>
+        <v/>
+      </c>
+      <c r="AH18">
+        <f>Settings!$B$2+AF18</f>
+        <v/>
+      </c>
+      <c r="AI18">
+        <f>AH18-AG18</f>
+        <v/>
+      </c>
+      <c r="AJ18">
+        <f>IF(OR(AND(C18&gt;0,W18=0),AND(E18&gt;0,Y18=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG18&gt;AH18,"ERROR: Rounded balance broken",IF(AI18&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -9775,6 +11427,34 @@
         <f>IF(AB19="FIXED","Close adjusted by SAFE mode",IF(AB19="SAFE","BUY/SELL balance preserved",IF(AB19="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD19">
+        <f>MAX(0,Settings!$B$2*G19/100-AA19)</f>
+        <v/>
+      </c>
+      <c r="AE19">
+        <f>SUM($W$3:W19)</f>
+        <v/>
+      </c>
+      <c r="AF19">
+        <f>SUM($Y$3:Y19)</f>
+        <v/>
+      </c>
+      <c r="AG19">
+        <f>AD19+AE19</f>
+        <v/>
+      </c>
+      <c r="AH19">
+        <f>Settings!$B$2+AF19</f>
+        <v/>
+      </c>
+      <c r="AI19">
+        <f>AH19-AG19</f>
+        <v/>
+      </c>
+      <c r="AJ19">
+        <f>IF(OR(AND(C19&gt;0,W19=0),AND(E19&gt;0,Y19=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG19&gt;AH19,"ERROR: Rounded balance broken",IF(AI19&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -9892,6 +11572,34 @@
         <f>IF(AB20="FIXED","Close adjusted by SAFE mode",IF(AB20="SAFE","BUY/SELL balance preserved",IF(AB20="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD20">
+        <f>MAX(0,Settings!$B$2*G20/100-AA20)</f>
+        <v/>
+      </c>
+      <c r="AE20">
+        <f>SUM($W$3:W20)</f>
+        <v/>
+      </c>
+      <c r="AF20">
+        <f>SUM($Y$3:Y20)</f>
+        <v/>
+      </c>
+      <c r="AG20">
+        <f>AD20+AE20</f>
+        <v/>
+      </c>
+      <c r="AH20">
+        <f>Settings!$B$2+AF20</f>
+        <v/>
+      </c>
+      <c r="AI20">
+        <f>AH20-AG20</f>
+        <v/>
+      </c>
+      <c r="AJ20">
+        <f>IF(OR(AND(C20&gt;0,W20=0),AND(E20&gt;0,Y20=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG20&gt;AH20,"ERROR: Rounded balance broken",IF(AI20&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -10009,6 +11717,34 @@
         <f>IF(AB21="FIXED","Close adjusted by SAFE mode",IF(AB21="SAFE","BUY/SELL balance preserved",IF(AB21="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD21">
+        <f>MAX(0,Settings!$B$2*G21/100-AA21)</f>
+        <v/>
+      </c>
+      <c r="AE21">
+        <f>SUM($W$3:W21)</f>
+        <v/>
+      </c>
+      <c r="AF21">
+        <f>SUM($Y$3:Y21)</f>
+        <v/>
+      </c>
+      <c r="AG21">
+        <f>AD21+AE21</f>
+        <v/>
+      </c>
+      <c r="AH21">
+        <f>Settings!$B$2+AF21</f>
+        <v/>
+      </c>
+      <c r="AI21">
+        <f>AH21-AG21</f>
+        <v/>
+      </c>
+      <c r="AJ21">
+        <f>IF(OR(AND(C21&gt;0,W21=0),AND(E21&gt;0,Y21=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG21&gt;AH21,"ERROR: Rounded balance broken",IF(AI21&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -10126,6 +11862,34 @@
         <f>IF(AB22="FIXED","Close adjusted by SAFE mode",IF(AB22="SAFE","BUY/SELL balance preserved",IF(AB22="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD22">
+        <f>MAX(0,Settings!$B$2*G22/100-AA22)</f>
+        <v/>
+      </c>
+      <c r="AE22">
+        <f>SUM($W$3:W22)</f>
+        <v/>
+      </c>
+      <c r="AF22">
+        <f>SUM($Y$3:Y22)</f>
+        <v/>
+      </c>
+      <c r="AG22">
+        <f>AD22+AE22</f>
+        <v/>
+      </c>
+      <c r="AH22">
+        <f>Settings!$B$2+AF22</f>
+        <v/>
+      </c>
+      <c r="AI22">
+        <f>AH22-AG22</f>
+        <v/>
+      </c>
+      <c r="AJ22">
+        <f>IF(OR(AND(C22&gt;0,W22=0),AND(E22&gt;0,Y22=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG22&gt;AH22,"ERROR: Rounded balance broken",IF(AI22&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -10243,6 +12007,34 @@
         <f>IF(AB23="FIXED","Close adjusted by SAFE mode",IF(AB23="SAFE","BUY/SELL balance preserved",IF(AB23="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD23">
+        <f>MAX(0,Settings!$B$2*G23/100-AA23)</f>
+        <v/>
+      </c>
+      <c r="AE23">
+        <f>SUM($W$3:W23)</f>
+        <v/>
+      </c>
+      <c r="AF23">
+        <f>SUM($Y$3:Y23)</f>
+        <v/>
+      </c>
+      <c r="AG23">
+        <f>AD23+AE23</f>
+        <v/>
+      </c>
+      <c r="AH23">
+        <f>Settings!$B$2+AF23</f>
+        <v/>
+      </c>
+      <c r="AI23">
+        <f>AH23-AG23</f>
+        <v/>
+      </c>
+      <c r="AJ23">
+        <f>IF(OR(AND(C23&gt;0,W23=0),AND(E23&gt;0,Y23=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG23&gt;AH23,"ERROR: Rounded balance broken",IF(AI23&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -10360,6 +12152,34 @@
         <f>IF(AB24="FIXED","Close adjusted by SAFE mode",IF(AB24="SAFE","BUY/SELL balance preserved",IF(AB24="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD24">
+        <f>MAX(0,Settings!$B$2*G24/100-AA24)</f>
+        <v/>
+      </c>
+      <c r="AE24">
+        <f>SUM($W$3:W24)</f>
+        <v/>
+      </c>
+      <c r="AF24">
+        <f>SUM($Y$3:Y24)</f>
+        <v/>
+      </c>
+      <c r="AG24">
+        <f>AD24+AE24</f>
+        <v/>
+      </c>
+      <c r="AH24">
+        <f>Settings!$B$2+AF24</f>
+        <v/>
+      </c>
+      <c r="AI24">
+        <f>AH24-AG24</f>
+        <v/>
+      </c>
+      <c r="AJ24">
+        <f>IF(OR(AND(C24&gt;0,W24=0),AND(E24&gt;0,Y24=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG24&gt;AH24,"ERROR: Rounded balance broken",IF(AI24&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -10477,6 +12297,34 @@
         <f>IF(AB25="FIXED","Close adjusted by SAFE mode",IF(AB25="SAFE","BUY/SELL balance preserved",IF(AB25="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD25">
+        <f>MAX(0,Settings!$B$2*G25/100-AA25)</f>
+        <v/>
+      </c>
+      <c r="AE25">
+        <f>SUM($W$3:W25)</f>
+        <v/>
+      </c>
+      <c r="AF25">
+        <f>SUM($Y$3:Y25)</f>
+        <v/>
+      </c>
+      <c r="AG25">
+        <f>AD25+AE25</f>
+        <v/>
+      </c>
+      <c r="AH25">
+        <f>Settings!$B$2+AF25</f>
+        <v/>
+      </c>
+      <c r="AI25">
+        <f>AH25-AG25</f>
+        <v/>
+      </c>
+      <c r="AJ25">
+        <f>IF(OR(AND(C25&gt;0,W25=0),AND(E25&gt;0,Y25=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG25&gt;AH25,"ERROR: Rounded balance broken",IF(AI25&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -10594,6 +12442,34 @@
         <f>IF(AB26="FIXED","Close adjusted by SAFE mode",IF(AB26="SAFE","BUY/SELL balance preserved",IF(AB26="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD26">
+        <f>MAX(0,Settings!$B$2*G26/100-AA26)</f>
+        <v/>
+      </c>
+      <c r="AE26">
+        <f>SUM($W$3:W26)</f>
+        <v/>
+      </c>
+      <c r="AF26">
+        <f>SUM($Y$3:Y26)</f>
+        <v/>
+      </c>
+      <c r="AG26">
+        <f>AD26+AE26</f>
+        <v/>
+      </c>
+      <c r="AH26">
+        <f>Settings!$B$2+AF26</f>
+        <v/>
+      </c>
+      <c r="AI26">
+        <f>AH26-AG26</f>
+        <v/>
+      </c>
+      <c r="AJ26">
+        <f>IF(OR(AND(C26&gt;0,W26=0),AND(E26&gt;0,Y26=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG26&gt;AH26,"ERROR: Rounded balance broken",IF(AI26&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -10711,6 +12587,34 @@
         <f>IF(AB27="FIXED","Close adjusted by SAFE mode",IF(AB27="SAFE","BUY/SELL balance preserved",IF(AB27="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD27">
+        <f>MAX(0,Settings!$B$2*G27/100-AA27)</f>
+        <v/>
+      </c>
+      <c r="AE27">
+        <f>SUM($W$3:W27)</f>
+        <v/>
+      </c>
+      <c r="AF27">
+        <f>SUM($Y$3:Y27)</f>
+        <v/>
+      </c>
+      <c r="AG27">
+        <f>AD27+AE27</f>
+        <v/>
+      </c>
+      <c r="AH27">
+        <f>Settings!$B$2+AF27</f>
+        <v/>
+      </c>
+      <c r="AI27">
+        <f>AH27-AG27</f>
+        <v/>
+      </c>
+      <c r="AJ27">
+        <f>IF(OR(AND(C27&gt;0,W27=0),AND(E27&gt;0,Y27=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG27&gt;AH27,"ERROR: Rounded balance broken",IF(AI27&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -10828,6 +12732,34 @@
         <f>IF(AB28="FIXED","Close adjusted by SAFE mode",IF(AB28="SAFE","BUY/SELL balance preserved",IF(AB28="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD28">
+        <f>MAX(0,Settings!$B$2*G28/100-AA28)</f>
+        <v/>
+      </c>
+      <c r="AE28">
+        <f>SUM($W$3:W28)</f>
+        <v/>
+      </c>
+      <c r="AF28">
+        <f>SUM($Y$3:Y28)</f>
+        <v/>
+      </c>
+      <c r="AG28">
+        <f>AD28+AE28</f>
+        <v/>
+      </c>
+      <c r="AH28">
+        <f>Settings!$B$2+AF28</f>
+        <v/>
+      </c>
+      <c r="AI28">
+        <f>AH28-AG28</f>
+        <v/>
+      </c>
+      <c r="AJ28">
+        <f>IF(OR(AND(C28&gt;0,W28=0),AND(E28&gt;0,Y28=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG28&gt;AH28,"ERROR: Rounded balance broken",IF(AI28&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -10945,6 +12877,34 @@
         <f>IF(AB29="FIXED","Close adjusted by SAFE mode",IF(AB29="SAFE","BUY/SELL balance preserved",IF(AB29="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD29">
+        <f>MAX(0,Settings!$B$2*G29/100-AA29)</f>
+        <v/>
+      </c>
+      <c r="AE29">
+        <f>SUM($W$3:W29)</f>
+        <v/>
+      </c>
+      <c r="AF29">
+        <f>SUM($Y$3:Y29)</f>
+        <v/>
+      </c>
+      <c r="AG29">
+        <f>AD29+AE29</f>
+        <v/>
+      </c>
+      <c r="AH29">
+        <f>Settings!$B$2+AF29</f>
+        <v/>
+      </c>
+      <c r="AI29">
+        <f>AH29-AG29</f>
+        <v/>
+      </c>
+      <c r="AJ29">
+        <f>IF(OR(AND(C29&gt;0,W29=0),AND(E29&gt;0,Y29=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG29&gt;AH29,"ERROR: Rounded balance broken",IF(AI29&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -11062,6 +13022,34 @@
         <f>IF(AB30="FIXED","Close adjusted by SAFE mode",IF(AB30="SAFE","BUY/SELL balance preserved",IF(AB30="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD30">
+        <f>MAX(0,Settings!$B$2*G30/100-AA30)</f>
+        <v/>
+      </c>
+      <c r="AE30">
+        <f>SUM($W$3:W30)</f>
+        <v/>
+      </c>
+      <c r="AF30">
+        <f>SUM($Y$3:Y30)</f>
+        <v/>
+      </c>
+      <c r="AG30">
+        <f>AD30+AE30</f>
+        <v/>
+      </c>
+      <c r="AH30">
+        <f>Settings!$B$2+AF30</f>
+        <v/>
+      </c>
+      <c r="AI30">
+        <f>AH30-AG30</f>
+        <v/>
+      </c>
+      <c r="AJ30">
+        <f>IF(OR(AND(C30&gt;0,W30=0),AND(E30&gt;0,Y30=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG30&gt;AH30,"ERROR: Rounded balance broken",IF(AI30&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -11179,6 +13167,34 @@
         <f>IF(AB31="FIXED","Close adjusted by SAFE mode",IF(AB31="SAFE","BUY/SELL balance preserved",IF(AB31="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD31">
+        <f>MAX(0,Settings!$B$2*G31/100-AA31)</f>
+        <v/>
+      </c>
+      <c r="AE31">
+        <f>SUM($W$3:W31)</f>
+        <v/>
+      </c>
+      <c r="AF31">
+        <f>SUM($Y$3:Y31)</f>
+        <v/>
+      </c>
+      <c r="AG31">
+        <f>AD31+AE31</f>
+        <v/>
+      </c>
+      <c r="AH31">
+        <f>Settings!$B$2+AF31</f>
+        <v/>
+      </c>
+      <c r="AI31">
+        <f>AH31-AG31</f>
+        <v/>
+      </c>
+      <c r="AJ31">
+        <f>IF(OR(AND(C31&gt;0,W31=0),AND(E31&gt;0,Y31=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG31&gt;AH31,"ERROR: Rounded balance broken",IF(AI31&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -11296,6 +13312,34 @@
         <f>IF(AB32="FIXED","Close adjusted by SAFE mode",IF(AB32="SAFE","BUY/SELL balance preserved",IF(AB32="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD32">
+        <f>MAX(0,Settings!$B$2*G32/100-AA32)</f>
+        <v/>
+      </c>
+      <c r="AE32">
+        <f>SUM($W$3:W32)</f>
+        <v/>
+      </c>
+      <c r="AF32">
+        <f>SUM($Y$3:Y32)</f>
+        <v/>
+      </c>
+      <c r="AG32">
+        <f>AD32+AE32</f>
+        <v/>
+      </c>
+      <c r="AH32">
+        <f>Settings!$B$2+AF32</f>
+        <v/>
+      </c>
+      <c r="AI32">
+        <f>AH32-AG32</f>
+        <v/>
+      </c>
+      <c r="AJ32">
+        <f>IF(OR(AND(C32&gt;0,W32=0),AND(E32&gt;0,Y32=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG32&gt;AH32,"ERROR: Rounded balance broken",IF(AI32&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -11413,6 +13457,34 @@
         <f>IF(AB33="FIXED","Close adjusted by SAFE mode",IF(AB33="SAFE","BUY/SELL balance preserved",IF(AB33="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD33">
+        <f>MAX(0,Settings!$B$2*G33/100-AA33)</f>
+        <v/>
+      </c>
+      <c r="AE33">
+        <f>SUM($W$3:W33)</f>
+        <v/>
+      </c>
+      <c r="AF33">
+        <f>SUM($Y$3:Y33)</f>
+        <v/>
+      </c>
+      <c r="AG33">
+        <f>AD33+AE33</f>
+        <v/>
+      </c>
+      <c r="AH33">
+        <f>Settings!$B$2+AF33</f>
+        <v/>
+      </c>
+      <c r="AI33">
+        <f>AH33-AG33</f>
+        <v/>
+      </c>
+      <c r="AJ33">
+        <f>IF(OR(AND(C33&gt;0,W33=0),AND(E33&gt;0,Y33=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG33&gt;AH33,"ERROR: Rounded balance broken",IF(AI33&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -11530,6 +13602,34 @@
         <f>IF(AB34="FIXED","Close adjusted by SAFE mode",IF(AB34="SAFE","BUY/SELL balance preserved",IF(AB34="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD34">
+        <f>MAX(0,Settings!$B$2*G34/100-AA34)</f>
+        <v/>
+      </c>
+      <c r="AE34">
+        <f>SUM($W$3:W34)</f>
+        <v/>
+      </c>
+      <c r="AF34">
+        <f>SUM($Y$3:Y34)</f>
+        <v/>
+      </c>
+      <c r="AG34">
+        <f>AD34+AE34</f>
+        <v/>
+      </c>
+      <c r="AH34">
+        <f>Settings!$B$2+AF34</f>
+        <v/>
+      </c>
+      <c r="AI34">
+        <f>AH34-AG34</f>
+        <v/>
+      </c>
+      <c r="AJ34">
+        <f>IF(OR(AND(C34&gt;0,W34=0),AND(E34&gt;0,Y34=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG34&gt;AH34,"ERROR: Rounded balance broken",IF(AI34&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -11647,6 +13747,34 @@
         <f>IF(AB35="FIXED","Close adjusted by SAFE mode",IF(AB35="SAFE","BUY/SELL balance preserved",IF(AB35="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD35">
+        <f>MAX(0,Settings!$B$2*G35/100-AA35)</f>
+        <v/>
+      </c>
+      <c r="AE35">
+        <f>SUM($W$3:W35)</f>
+        <v/>
+      </c>
+      <c r="AF35">
+        <f>SUM($Y$3:Y35)</f>
+        <v/>
+      </c>
+      <c r="AG35">
+        <f>AD35+AE35</f>
+        <v/>
+      </c>
+      <c r="AH35">
+        <f>Settings!$B$2+AF35</f>
+        <v/>
+      </c>
+      <c r="AI35">
+        <f>AH35-AG35</f>
+        <v/>
+      </c>
+      <c r="AJ35">
+        <f>IF(OR(AND(C35&gt;0,W35=0),AND(E35&gt;0,Y35=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG35&gt;AH35,"ERROR: Rounded balance broken",IF(AI35&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -11764,6 +13892,34 @@
         <f>IF(AB36="FIXED","Close adjusted by SAFE mode",IF(AB36="SAFE","BUY/SELL balance preserved",IF(AB36="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD36">
+        <f>MAX(0,Settings!$B$2*G36/100-AA36)</f>
+        <v/>
+      </c>
+      <c r="AE36">
+        <f>SUM($W$3:W36)</f>
+        <v/>
+      </c>
+      <c r="AF36">
+        <f>SUM($Y$3:Y36)</f>
+        <v/>
+      </c>
+      <c r="AG36">
+        <f>AD36+AE36</f>
+        <v/>
+      </c>
+      <c r="AH36">
+        <f>Settings!$B$2+AF36</f>
+        <v/>
+      </c>
+      <c r="AI36">
+        <f>AH36-AG36</f>
+        <v/>
+      </c>
+      <c r="AJ36">
+        <f>IF(OR(AND(C36&gt;0,W36=0),AND(E36&gt;0,Y36=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG36&gt;AH36,"ERROR: Rounded balance broken",IF(AI36&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -11881,6 +14037,34 @@
         <f>IF(AB37="FIXED","Close adjusted by SAFE mode",IF(AB37="SAFE","BUY/SELL balance preserved",IF(AB37="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD37">
+        <f>MAX(0,Settings!$B$2*G37/100-AA37)</f>
+        <v/>
+      </c>
+      <c r="AE37">
+        <f>SUM($W$3:W37)</f>
+        <v/>
+      </c>
+      <c r="AF37">
+        <f>SUM($Y$3:Y37)</f>
+        <v/>
+      </c>
+      <c r="AG37">
+        <f>AD37+AE37</f>
+        <v/>
+      </c>
+      <c r="AH37">
+        <f>Settings!$B$2+AF37</f>
+        <v/>
+      </c>
+      <c r="AI37">
+        <f>AH37-AG37</f>
+        <v/>
+      </c>
+      <c r="AJ37">
+        <f>IF(OR(AND(C37&gt;0,W37=0),AND(E37&gt;0,Y37=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG37&gt;AH37,"ERROR: Rounded balance broken",IF(AI37&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -11998,6 +14182,34 @@
         <f>IF(AB38="FIXED","Close adjusted by SAFE mode",IF(AB38="SAFE","BUY/SELL balance preserved",IF(AB38="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD38">
+        <f>MAX(0,Settings!$B$2*G38/100-AA38)</f>
+        <v/>
+      </c>
+      <c r="AE38">
+        <f>SUM($W$3:W38)</f>
+        <v/>
+      </c>
+      <c r="AF38">
+        <f>SUM($Y$3:Y38)</f>
+        <v/>
+      </c>
+      <c r="AG38">
+        <f>AD38+AE38</f>
+        <v/>
+      </c>
+      <c r="AH38">
+        <f>Settings!$B$2+AF38</f>
+        <v/>
+      </c>
+      <c r="AI38">
+        <f>AH38-AG38</f>
+        <v/>
+      </c>
+      <c r="AJ38">
+        <f>IF(OR(AND(C38&gt;0,W38=0),AND(E38&gt;0,Y38=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG38&gt;AH38,"ERROR: Rounded balance broken",IF(AI38&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -12115,6 +14327,34 @@
         <f>IF(AB39="FIXED","Close adjusted by SAFE mode",IF(AB39="SAFE","BUY/SELL balance preserved",IF(AB39="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD39">
+        <f>MAX(0,Settings!$B$2*G39/100-AA39)</f>
+        <v/>
+      </c>
+      <c r="AE39">
+        <f>SUM($W$3:W39)</f>
+        <v/>
+      </c>
+      <c r="AF39">
+        <f>SUM($Y$3:Y39)</f>
+        <v/>
+      </c>
+      <c r="AG39">
+        <f>AD39+AE39</f>
+        <v/>
+      </c>
+      <c r="AH39">
+        <f>Settings!$B$2+AF39</f>
+        <v/>
+      </c>
+      <c r="AI39">
+        <f>AH39-AG39</f>
+        <v/>
+      </c>
+      <c r="AJ39">
+        <f>IF(OR(AND(C39&gt;0,W39=0),AND(E39&gt;0,Y39=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG39&gt;AH39,"ERROR: Rounded balance broken",IF(AI39&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -12232,6 +14472,34 @@
         <f>IF(AB40="FIXED","Close adjusted by SAFE mode",IF(AB40="SAFE","BUY/SELL balance preserved",IF(AB40="WARNING","Near protection boundary","Protection broken")))</f>
         <v/>
       </c>
+      <c r="AD40">
+        <f>MAX(0,Settings!$B$2*G40/100-AA40)</f>
+        <v/>
+      </c>
+      <c r="AE40">
+        <f>SUM($W$3:W40)</f>
+        <v/>
+      </c>
+      <c r="AF40">
+        <f>SUM($Y$3:Y40)</f>
+        <v/>
+      </c>
+      <c r="AG40">
+        <f>AD40+AE40</f>
+        <v/>
+      </c>
+      <c r="AH40">
+        <f>Settings!$B$2+AF40</f>
+        <v/>
+      </c>
+      <c r="AI40">
+        <f>AH40-AG40</f>
+        <v/>
+      </c>
+      <c r="AJ40">
+        <f>IF(OR(AND(C40&gt;0,W40=0),AND(E40&gt;0,Y40=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG40&gt;AH40,"ERROR: Rounded balance broken",IF(AI40&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -12347,6 +14615,34 @@
       </c>
       <c r="AC41">
         <f>IF(AB41="FIXED","Close adjusted by SAFE mode",IF(AB41="SAFE","BUY/SELL balance preserved",IF(AB41="WARNING","Near protection boundary","Protection broken")))</f>
+        <v/>
+      </c>
+      <c r="AD41">
+        <f>MAX(0,Settings!$B$2*G41/100-AA41)</f>
+        <v/>
+      </c>
+      <c r="AE41">
+        <f>SUM($W$3:W41)</f>
+        <v/>
+      </c>
+      <c r="AF41">
+        <f>SUM($Y$3:Y41)</f>
+        <v/>
+      </c>
+      <c r="AG41">
+        <f>AD41+AE41</f>
+        <v/>
+      </c>
+      <c r="AH41">
+        <f>Settings!$B$2+AF41</f>
+        <v/>
+      </c>
+      <c r="AI41">
+        <f>AH41-AG41</f>
+        <v/>
+      </c>
+      <c r="AJ41">
+        <f>IF(OR(AND(C41&gt;0,W41=0),AND(E41&gt;0,Y41=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG41&gt;AH41,"ERROR: Rounded balance broken",IF(AI41&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -12375,7 +14671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12410,66 +14706,132 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Adaptive Step</t>
+          <t>Final Total BUY %</t>
         </is>
       </c>
       <c r="B5">
-        <f>MarketModel!B16</f>
+        <f>INDEX(DownTrend!Q:Q,Settings!B4+3)</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ATR Regime</t>
+          <t>Final Total SELL %</t>
         </is>
       </c>
       <c r="B6">
-        <f>MarketModel!B11</f>
+        <f>INDEX(DownTrend!R:R,Settings!B4+3)</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Margin Load</t>
+          <t>Final Skew %</t>
         </is>
       </c>
       <c r="B7">
-        <f>MarginControl!B13</f>
+        <f>INDEX(DownTrend!S:S,Settings!B4+3)</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Risk Score</t>
+          <t>Final id1 Remaining %</t>
         </is>
       </c>
       <c r="B8">
-        <f>RiskDashboard!B4</f>
+        <f>INDEX(DownTrend!N:N,Settings!B4+3)</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Max Safe Levels</t>
+          <t>Adaptive Step</t>
         </is>
       </c>
       <c r="B9">
-        <f>MarginControl!B17</f>
+        <f>MarketModel!B16</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>ATR Regime</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>MarketModel!B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Margin Load</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>MarginControl!B13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Risk Score</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>RiskDashboard!B4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Risk Status</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>RiskDashboard!B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Survival Probability</t>
         </is>
       </c>
-      <c r="B10">
+      <c r="B14">
         <f>RiskDashboard!B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Final System Status</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>IF(COUNTIF(DownTrend!T3:INDEX(DownTrend!T:T,Settings!B4+3),"ERROR*")+COUNTIF(UpTrend!T3:INDEX(UpTrend!T:T,Settings!B4+3),"ERROR*")&gt;0,"ERROR",IF(COUNTIF(DownTrend!T3:INDEX(DownTrend!T:T,Settings!B4+3),"WARNING*")+COUNTIF(UpTrend!T3:INDEX(UpTrend!T:T,Settings!B4+3),"WARNING*")&gt;0,"WARNING","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Rounded System Status</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>IF(COUNTIF(DownTrend!AJ3:INDEX(DownTrend!AJ:AJ,Settings!B4+3),"ERROR*")+COUNTIF(UpTrend!AJ3:INDEX(UpTrend!AJ:AJ,Settings!B4+3),"ERROR*")&gt;0,"ERROR",IF(COUNTIF(DownTrend!AJ3:INDEX(DownTrend!AJ:AJ,Settings!B4+3),"WARNING*")+COUNTIF(UpTrend!AJ3:INDEX(UpTrend!AJ:AJ,Settings!B4+3),"WARNING*")&gt;0,"WARNING","OK"))</f>
         <v/>
       </c>
     </row>
@@ -12485,7 +14847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12498,77 +14860,143 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Big&gt;=Small</t>
+          <t>Invalid StartLot</t>
         </is>
       </c>
       <c r="B2">
-        <f>IF(SUMPRODUCT(--(DownTrend!C3:C41&lt;DownTrend!E3:E41))+SUMPRODUCT(--(UpTrend!C3:C41&lt;UpTrend!E3:E41))&gt;0,"ERROR","OK")</f>
+        <f>IF(OR(NOT(ISNUMBER(Settings!B2)),Settings!B2&lt;=0),"ERROR","OK")</f>
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TotalBUY&lt;=TotalSELL Down</t>
+          <t>Invalid LotStep</t>
         </is>
       </c>
       <c r="B3">
-        <f>IF(SUMPRODUCT(--(DownTrend!Q3:Q41&gt;DownTrend!R3:R41))&gt;0,"ERROR","OK")</f>
+        <f>IF(OR(NOT(ISNUMBER(Settings!B5)),Settings!B5&lt;=0),"ERROR","OK")</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TotalSELL&lt;=TotalBUY Up</t>
+          <t>Invalid Direction</t>
         </is>
       </c>
       <c r="B4">
-        <f>IF(SUMPRODUCT(--(UpTrend!Q3:Q41&gt;UpTrend!R3:R41))&gt;0,"ERROR","OK")</f>
+        <f>IF(AND(Settings!B10&lt;&gt;"DOWN",Settings!B10&lt;&gt;"UP"),"ERROR","OK")</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SAFE rounding preserved</t>
+          <t>Negative values</t>
         </is>
       </c>
       <c r="B5">
-        <f>IF(OR(COUNTIF(DownTrend!AB3:AB41,"ERROR")&gt;0,COUNTIF(UpTrend!AB3:AB41,"ERROR")&gt;0),"ERROR","OK")</f>
+        <f>IF(OR(MIN(Settings!B22:E200)&lt;0,MIN(DownTrend!N3:N41)&lt;0,MIN(UpTrend!N3:N41)&lt;0),"ERROR","OK")</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Invalid StartLot</t>
+          <t>Big &lt; Small</t>
         </is>
       </c>
       <c r="B6">
-        <f>IF(OR(NOT(ISNUMBER(Settings!B2)),Settings!B2&lt;=0),"ERROR","OK")</f>
+        <f>IF(SUMPRODUCT(--(DownTrend!C3:C41&lt;DownTrend!E3:E41))+SUMPRODUCT(--(UpTrend!C3:C41&lt;UpTrend!E3:E41))&gt;0,"ERROR","OK")</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Invalid LotStep</t>
+          <t>ManualClose &gt; Remaining</t>
         </is>
       </c>
       <c r="B7">
-        <f>IF(OR(NOT(ISNUMBER(Settings!B5)),Settings!B5&lt;=0),"ERROR","OK")</f>
+        <f>IF(OR(SUMPRODUCT(--(DownTrend!L3:L41&gt;DownTrend!G3:G41))&gt;0,SUMPRODUCT(--(UpTrend!L3:L41&gt;UpTrend!G3:G41))&gt;0),"ERROR","OK")</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Invalid Direction</t>
+          <t>Remaining &lt; 0</t>
         </is>
       </c>
       <c r="B8">
-        <f>IF(AND(Settings!B10&lt;&gt;"DOWN",Settings!B10&lt;&gt;"UP"),"ERROR","OK")</f>
+        <f>IF(OR(MIN(DownTrend!N3:N41)&lt;0,MIN(UpTrend!N3:N41)&lt;0),"ERROR","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Protection balance</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>IF(OR(SUMPRODUCT(--(DownTrend!Q3:Q41&gt;DownTrend!R3:R41))&gt;0,SUMPRODUCT(--(UpTrend!Q3:Q41&gt;UpTrend!R3:R41))&gt;0),"ERROR","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Rounded safety preserved</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>IF(OR(COUNTIF(DownTrend!AJ3:AJ41,"ERROR*")&gt;0,COUNTIF(UpTrend!AJ3:AJ41,"ERROR*")&gt;0),"ERROR","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Rounded Big zero</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>IF(OR(SUMPRODUCT(--(DownTrend!C3:C41&gt;0),--(DownTrend!W3:W41=0))&gt;0,SUMPRODUCT(--(UpTrend!C3:C41&gt;0),--(UpTrend!W3:W41=0))&gt;0),"ERROR","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Rounded Small zero</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>IF(OR(SUMPRODUCT(--(DownTrend!E3:E41&gt;0),--(DownTrend!Y3:Y41=0))&gt;0,SUMPRODUCT(--(UpTrend!E3:E41&gt;0),--(UpTrend!Y3:Y41=0))&gt;0),"ERROR","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>LotStep too coarse</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>IF(Settings!B2&lt;Settings!B5,"ERROR","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>FinalStatus from T/AJ</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>IF(OR(COUNTIF(DownTrend!T3:T41,"ERROR*")&gt;0,COUNTIF(UpTrend!T3:T41,"ERROR*")&gt;0,COUNTIF(DownTrend!AJ3:AJ41,"ERROR*")&gt;0,COUNTIF(UpTrend!AJ3:AJ41,"ERROR*")&gt;0),"ERROR",IF(OR(COUNTIF(DownTrend!T3:T41,"WARNING*")&gt;0,COUNTIF(UpTrend!T3:T41,"WARNING*")&gt;0,COUNTIF(DownTrend!AJ3:AJ41,"WARNING*")&gt;0,COUNTIF(UpTrend!AJ3:AJ41,"WARNING*")&gt;0),"WARNING","OK"))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix AJ baseline warning and Summary direction switch
</commit_message>
<xml_diff>
--- a/MinusLock_Percent_Grid_Calculator/MinusLock_Percent_Grid_Calculator.xlsx
+++ b/MinusLock_Percent_Grid_Calculator/MinusLock_Percent_Grid_Calculator.xlsx
@@ -3151,7 +3151,7 @@
         <v/>
       </c>
       <c r="AJ3">
-        <f>IF(OR(AND(C3&gt;0,W3=0),AND(E3&gt;0,Y3=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG3&gt;AH3,"ERROR: Rounded balance broken",IF(AI3&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C3&gt;0,W3=0),AND(E3&gt;0,Y3=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG3&gt;AH3,"ERROR: Rounded balance broken",IF(AND(J3&gt;0,AI3&lt;Settings!$B$2*J3/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -3296,7 +3296,7 @@
         <v/>
       </c>
       <c r="AJ4">
-        <f>IF(OR(AND(C4&gt;0,W4=0),AND(E4&gt;0,Y4=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG4&gt;AH4,"ERROR: Rounded balance broken",IF(AI4&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C4&gt;0,W4=0),AND(E4&gt;0,Y4=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG4&gt;AH4,"ERROR: Rounded balance broken",IF(AND(J4&gt;0,AI4&lt;Settings!$B$2*J4/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -3441,7 +3441,7 @@
         <v/>
       </c>
       <c r="AJ5">
-        <f>IF(OR(AND(C5&gt;0,W5=0),AND(E5&gt;0,Y5=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG5&gt;AH5,"ERROR: Rounded balance broken",IF(AI5&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C5&gt;0,W5=0),AND(E5&gt;0,Y5=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG5&gt;AH5,"ERROR: Rounded balance broken",IF(AND(J5&gt;0,AI5&lt;Settings!$B$2*J5/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -3586,7 +3586,7 @@
         <v/>
       </c>
       <c r="AJ6">
-        <f>IF(OR(AND(C6&gt;0,W6=0),AND(E6&gt;0,Y6=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG6&gt;AH6,"ERROR: Rounded balance broken",IF(AI6&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C6&gt;0,W6=0),AND(E6&gt;0,Y6=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG6&gt;AH6,"ERROR: Rounded balance broken",IF(AND(J6&gt;0,AI6&lt;Settings!$B$2*J6/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -3731,7 +3731,7 @@
         <v/>
       </c>
       <c r="AJ7">
-        <f>IF(OR(AND(C7&gt;0,W7=0),AND(E7&gt;0,Y7=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG7&gt;AH7,"ERROR: Rounded balance broken",IF(AI7&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C7&gt;0,W7=0),AND(E7&gt;0,Y7=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG7&gt;AH7,"ERROR: Rounded balance broken",IF(AND(J7&gt;0,AI7&lt;Settings!$B$2*J7/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -3876,7 +3876,7 @@
         <v/>
       </c>
       <c r="AJ8">
-        <f>IF(OR(AND(C8&gt;0,W8=0),AND(E8&gt;0,Y8=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG8&gt;AH8,"ERROR: Rounded balance broken",IF(AI8&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C8&gt;0,W8=0),AND(E8&gt;0,Y8=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG8&gt;AH8,"ERROR: Rounded balance broken",IF(AND(J8&gt;0,AI8&lt;Settings!$B$2*J8/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -4021,7 +4021,7 @@
         <v/>
       </c>
       <c r="AJ9">
-        <f>IF(OR(AND(C9&gt;0,W9=0),AND(E9&gt;0,Y9=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG9&gt;AH9,"ERROR: Rounded balance broken",IF(AI9&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C9&gt;0,W9=0),AND(E9&gt;0,Y9=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG9&gt;AH9,"ERROR: Rounded balance broken",IF(AND(J9&gt;0,AI9&lt;Settings!$B$2*J9/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -4166,7 +4166,7 @@
         <v/>
       </c>
       <c r="AJ10">
-        <f>IF(OR(AND(C10&gt;0,W10=0),AND(E10&gt;0,Y10=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG10&gt;AH10,"ERROR: Rounded balance broken",IF(AI10&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C10&gt;0,W10=0),AND(E10&gt;0,Y10=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG10&gt;AH10,"ERROR: Rounded balance broken",IF(AND(J10&gt;0,AI10&lt;Settings!$B$2*J10/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -4311,7 +4311,7 @@
         <v/>
       </c>
       <c r="AJ11">
-        <f>IF(OR(AND(C11&gt;0,W11=0),AND(E11&gt;0,Y11=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG11&gt;AH11,"ERROR: Rounded balance broken",IF(AI11&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C11&gt;0,W11=0),AND(E11&gt;0,Y11=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG11&gt;AH11,"ERROR: Rounded balance broken",IF(AND(J11&gt;0,AI11&lt;Settings!$B$2*J11/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -4456,7 +4456,7 @@
         <v/>
       </c>
       <c r="AJ12">
-        <f>IF(OR(AND(C12&gt;0,W12=0),AND(E12&gt;0,Y12=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG12&gt;AH12,"ERROR: Rounded balance broken",IF(AI12&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C12&gt;0,W12=0),AND(E12&gt;0,Y12=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG12&gt;AH12,"ERROR: Rounded balance broken",IF(AND(J12&gt;0,AI12&lt;Settings!$B$2*J12/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -4601,7 +4601,7 @@
         <v/>
       </c>
       <c r="AJ13">
-        <f>IF(OR(AND(C13&gt;0,W13=0),AND(E13&gt;0,Y13=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG13&gt;AH13,"ERROR: Rounded balance broken",IF(AI13&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C13&gt;0,W13=0),AND(E13&gt;0,Y13=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG13&gt;AH13,"ERROR: Rounded balance broken",IF(AND(J13&gt;0,AI13&lt;Settings!$B$2*J13/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -4746,7 +4746,7 @@
         <v/>
       </c>
       <c r="AJ14">
-        <f>IF(OR(AND(C14&gt;0,W14=0),AND(E14&gt;0,Y14=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG14&gt;AH14,"ERROR: Rounded balance broken",IF(AI14&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C14&gt;0,W14=0),AND(E14&gt;0,Y14=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG14&gt;AH14,"ERROR: Rounded balance broken",IF(AND(J14&gt;0,AI14&lt;Settings!$B$2*J14/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -4891,7 +4891,7 @@
         <v/>
       </c>
       <c r="AJ15">
-        <f>IF(OR(AND(C15&gt;0,W15=0),AND(E15&gt;0,Y15=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG15&gt;AH15,"ERROR: Rounded balance broken",IF(AI15&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C15&gt;0,W15=0),AND(E15&gt;0,Y15=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG15&gt;AH15,"ERROR: Rounded balance broken",IF(AND(J15&gt;0,AI15&lt;Settings!$B$2*J15/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -5036,7 +5036,7 @@
         <v/>
       </c>
       <c r="AJ16">
-        <f>IF(OR(AND(C16&gt;0,W16=0),AND(E16&gt;0,Y16=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG16&gt;AH16,"ERROR: Rounded balance broken",IF(AI16&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C16&gt;0,W16=0),AND(E16&gt;0,Y16=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG16&gt;AH16,"ERROR: Rounded balance broken",IF(AND(J16&gt;0,AI16&lt;Settings!$B$2*J16/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -5181,7 +5181,7 @@
         <v/>
       </c>
       <c r="AJ17">
-        <f>IF(OR(AND(C17&gt;0,W17=0),AND(E17&gt;0,Y17=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG17&gt;AH17,"ERROR: Rounded balance broken",IF(AI17&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C17&gt;0,W17=0),AND(E17&gt;0,Y17=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG17&gt;AH17,"ERROR: Rounded balance broken",IF(AND(J17&gt;0,AI17&lt;Settings!$B$2*J17/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -5326,7 +5326,7 @@
         <v/>
       </c>
       <c r="AJ18">
-        <f>IF(OR(AND(C18&gt;0,W18=0),AND(E18&gt;0,Y18=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG18&gt;AH18,"ERROR: Rounded balance broken",IF(AI18&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C18&gt;0,W18=0),AND(E18&gt;0,Y18=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG18&gt;AH18,"ERROR: Rounded balance broken",IF(AND(J18&gt;0,AI18&lt;Settings!$B$2*J18/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -5471,7 +5471,7 @@
         <v/>
       </c>
       <c r="AJ19">
-        <f>IF(OR(AND(C19&gt;0,W19=0),AND(E19&gt;0,Y19=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG19&gt;AH19,"ERROR: Rounded balance broken",IF(AI19&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C19&gt;0,W19=0),AND(E19&gt;0,Y19=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG19&gt;AH19,"ERROR: Rounded balance broken",IF(AND(J19&gt;0,AI19&lt;Settings!$B$2*J19/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
         <v/>
       </c>
       <c r="AJ20">
-        <f>IF(OR(AND(C20&gt;0,W20=0),AND(E20&gt;0,Y20=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG20&gt;AH20,"ERROR: Rounded balance broken",IF(AI20&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C20&gt;0,W20=0),AND(E20&gt;0,Y20=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG20&gt;AH20,"ERROR: Rounded balance broken",IF(AND(J20&gt;0,AI20&lt;Settings!$B$2*J20/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -5761,7 +5761,7 @@
         <v/>
       </c>
       <c r="AJ21">
-        <f>IF(OR(AND(C21&gt;0,W21=0),AND(E21&gt;0,Y21=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG21&gt;AH21,"ERROR: Rounded balance broken",IF(AI21&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C21&gt;0,W21=0),AND(E21&gt;0,Y21=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG21&gt;AH21,"ERROR: Rounded balance broken",IF(AND(J21&gt;0,AI21&lt;Settings!$B$2*J21/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -5906,7 +5906,7 @@
         <v/>
       </c>
       <c r="AJ22">
-        <f>IF(OR(AND(C22&gt;0,W22=0),AND(E22&gt;0,Y22=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG22&gt;AH22,"ERROR: Rounded balance broken",IF(AI22&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C22&gt;0,W22=0),AND(E22&gt;0,Y22=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG22&gt;AH22,"ERROR: Rounded balance broken",IF(AND(J22&gt;0,AI22&lt;Settings!$B$2*J22/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -6051,7 +6051,7 @@
         <v/>
       </c>
       <c r="AJ23">
-        <f>IF(OR(AND(C23&gt;0,W23=0),AND(E23&gt;0,Y23=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG23&gt;AH23,"ERROR: Rounded balance broken",IF(AI23&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C23&gt;0,W23=0),AND(E23&gt;0,Y23=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG23&gt;AH23,"ERROR: Rounded balance broken",IF(AND(J23&gt;0,AI23&lt;Settings!$B$2*J23/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -6196,7 +6196,7 @@
         <v/>
       </c>
       <c r="AJ24">
-        <f>IF(OR(AND(C24&gt;0,W24=0),AND(E24&gt;0,Y24=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG24&gt;AH24,"ERROR: Rounded balance broken",IF(AI24&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C24&gt;0,W24=0),AND(E24&gt;0,Y24=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG24&gt;AH24,"ERROR: Rounded balance broken",IF(AND(J24&gt;0,AI24&lt;Settings!$B$2*J24/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -6341,7 +6341,7 @@
         <v/>
       </c>
       <c r="AJ25">
-        <f>IF(OR(AND(C25&gt;0,W25=0),AND(E25&gt;0,Y25=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG25&gt;AH25,"ERROR: Rounded balance broken",IF(AI25&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C25&gt;0,W25=0),AND(E25&gt;0,Y25=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG25&gt;AH25,"ERROR: Rounded balance broken",IF(AND(J25&gt;0,AI25&lt;Settings!$B$2*J25/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -6486,7 +6486,7 @@
         <v/>
       </c>
       <c r="AJ26">
-        <f>IF(OR(AND(C26&gt;0,W26=0),AND(E26&gt;0,Y26=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG26&gt;AH26,"ERROR: Rounded balance broken",IF(AI26&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C26&gt;0,W26=0),AND(E26&gt;0,Y26=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG26&gt;AH26,"ERROR: Rounded balance broken",IF(AND(J26&gt;0,AI26&lt;Settings!$B$2*J26/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -6631,7 +6631,7 @@
         <v/>
       </c>
       <c r="AJ27">
-        <f>IF(OR(AND(C27&gt;0,W27=0),AND(E27&gt;0,Y27=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG27&gt;AH27,"ERROR: Rounded balance broken",IF(AI27&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C27&gt;0,W27=0),AND(E27&gt;0,Y27=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG27&gt;AH27,"ERROR: Rounded balance broken",IF(AND(J27&gt;0,AI27&lt;Settings!$B$2*J27/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -6776,7 +6776,7 @@
         <v/>
       </c>
       <c r="AJ28">
-        <f>IF(OR(AND(C28&gt;0,W28=0),AND(E28&gt;0,Y28=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG28&gt;AH28,"ERROR: Rounded balance broken",IF(AI28&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C28&gt;0,W28=0),AND(E28&gt;0,Y28=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG28&gt;AH28,"ERROR: Rounded balance broken",IF(AND(J28&gt;0,AI28&lt;Settings!$B$2*J28/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -6921,7 +6921,7 @@
         <v/>
       </c>
       <c r="AJ29">
-        <f>IF(OR(AND(C29&gt;0,W29=0),AND(E29&gt;0,Y29=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG29&gt;AH29,"ERROR: Rounded balance broken",IF(AI29&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C29&gt;0,W29=0),AND(E29&gt;0,Y29=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG29&gt;AH29,"ERROR: Rounded balance broken",IF(AND(J29&gt;0,AI29&lt;Settings!$B$2*J29/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -7066,7 +7066,7 @@
         <v/>
       </c>
       <c r="AJ30">
-        <f>IF(OR(AND(C30&gt;0,W30=0),AND(E30&gt;0,Y30=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG30&gt;AH30,"ERROR: Rounded balance broken",IF(AI30&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C30&gt;0,W30=0),AND(E30&gt;0,Y30=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG30&gt;AH30,"ERROR: Rounded balance broken",IF(AND(J30&gt;0,AI30&lt;Settings!$B$2*J30/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -7211,7 +7211,7 @@
         <v/>
       </c>
       <c r="AJ31">
-        <f>IF(OR(AND(C31&gt;0,W31=0),AND(E31&gt;0,Y31=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG31&gt;AH31,"ERROR: Rounded balance broken",IF(AI31&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C31&gt;0,W31=0),AND(E31&gt;0,Y31=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG31&gt;AH31,"ERROR: Rounded balance broken",IF(AND(J31&gt;0,AI31&lt;Settings!$B$2*J31/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -7356,7 +7356,7 @@
         <v/>
       </c>
       <c r="AJ32">
-        <f>IF(OR(AND(C32&gt;0,W32=0),AND(E32&gt;0,Y32=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG32&gt;AH32,"ERROR: Rounded balance broken",IF(AI32&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C32&gt;0,W32=0),AND(E32&gt;0,Y32=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG32&gt;AH32,"ERROR: Rounded balance broken",IF(AND(J32&gt;0,AI32&lt;Settings!$B$2*J32/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -7501,7 +7501,7 @@
         <v/>
       </c>
       <c r="AJ33">
-        <f>IF(OR(AND(C33&gt;0,W33=0),AND(E33&gt;0,Y33=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG33&gt;AH33,"ERROR: Rounded balance broken",IF(AI33&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C33&gt;0,W33=0),AND(E33&gt;0,Y33=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG33&gt;AH33,"ERROR: Rounded balance broken",IF(AND(J33&gt;0,AI33&lt;Settings!$B$2*J33/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -7646,7 +7646,7 @@
         <v/>
       </c>
       <c r="AJ34">
-        <f>IF(OR(AND(C34&gt;0,W34=0),AND(E34&gt;0,Y34=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG34&gt;AH34,"ERROR: Rounded balance broken",IF(AI34&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C34&gt;0,W34=0),AND(E34&gt;0,Y34=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG34&gt;AH34,"ERROR: Rounded balance broken",IF(AND(J34&gt;0,AI34&lt;Settings!$B$2*J34/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -7791,7 +7791,7 @@
         <v/>
       </c>
       <c r="AJ35">
-        <f>IF(OR(AND(C35&gt;0,W35=0),AND(E35&gt;0,Y35=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG35&gt;AH35,"ERROR: Rounded balance broken",IF(AI35&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C35&gt;0,W35=0),AND(E35&gt;0,Y35=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG35&gt;AH35,"ERROR: Rounded balance broken",IF(AND(J35&gt;0,AI35&lt;Settings!$B$2*J35/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -7936,7 +7936,7 @@
         <v/>
       </c>
       <c r="AJ36">
-        <f>IF(OR(AND(C36&gt;0,W36=0),AND(E36&gt;0,Y36=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG36&gt;AH36,"ERROR: Rounded balance broken",IF(AI36&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C36&gt;0,W36=0),AND(E36&gt;0,Y36=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG36&gt;AH36,"ERROR: Rounded balance broken",IF(AND(J36&gt;0,AI36&lt;Settings!$B$2*J36/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -8081,7 +8081,7 @@
         <v/>
       </c>
       <c r="AJ37">
-        <f>IF(OR(AND(C37&gt;0,W37=0),AND(E37&gt;0,Y37=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG37&gt;AH37,"ERROR: Rounded balance broken",IF(AI37&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C37&gt;0,W37=0),AND(E37&gt;0,Y37=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG37&gt;AH37,"ERROR: Rounded balance broken",IF(AND(J37&gt;0,AI37&lt;Settings!$B$2*J37/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -8226,7 +8226,7 @@
         <v/>
       </c>
       <c r="AJ38">
-        <f>IF(OR(AND(C38&gt;0,W38=0),AND(E38&gt;0,Y38=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG38&gt;AH38,"ERROR: Rounded balance broken",IF(AI38&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C38&gt;0,W38=0),AND(E38&gt;0,Y38=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG38&gt;AH38,"ERROR: Rounded balance broken",IF(AND(J38&gt;0,AI38&lt;Settings!$B$2*J38/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -8371,7 +8371,7 @@
         <v/>
       </c>
       <c r="AJ39">
-        <f>IF(OR(AND(C39&gt;0,W39=0),AND(E39&gt;0,Y39=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG39&gt;AH39,"ERROR: Rounded balance broken",IF(AI39&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C39&gt;0,W39=0),AND(E39&gt;0,Y39=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG39&gt;AH39,"ERROR: Rounded balance broken",IF(AND(J39&gt;0,AI39&lt;Settings!$B$2*J39/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -8516,7 +8516,7 @@
         <v/>
       </c>
       <c r="AJ40">
-        <f>IF(OR(AND(C40&gt;0,W40=0),AND(E40&gt;0,Y40=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG40&gt;AH40,"ERROR: Rounded balance broken",IF(AI40&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C40&gt;0,W40=0),AND(E40&gt;0,Y40=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG40&gt;AH40,"ERROR: Rounded balance broken",IF(AND(J40&gt;0,AI40&lt;Settings!$B$2*J40/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -8661,7 +8661,7 @@
         <v/>
       </c>
       <c r="AJ41">
-        <f>IF(OR(AND(C41&gt;0,W41=0),AND(E41&gt;0,Y41=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG41&gt;AH41,"ERROR: Rounded balance broken",IF(AI41&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C41&gt;0,W41=0),AND(E41&gt;0,Y41=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG41&gt;AH41,"ERROR: Rounded balance broken",IF(AND(J41&gt;0,AI41&lt;Settings!$B$2*J41/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -9132,7 +9132,7 @@
         <v/>
       </c>
       <c r="AJ3">
-        <f>IF(OR(AND(C3&gt;0,W3=0),AND(E3&gt;0,Y3=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG3&gt;AH3,"ERROR: Rounded balance broken",IF(AI3&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C3&gt;0,W3=0),AND(E3&gt;0,Y3=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG3&gt;AH3,"ERROR: Rounded balance broken",IF(AND(J3&gt;0,AI3&lt;Settings!$B$2*J3/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -9277,7 +9277,7 @@
         <v/>
       </c>
       <c r="AJ4">
-        <f>IF(OR(AND(C4&gt;0,W4=0),AND(E4&gt;0,Y4=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG4&gt;AH4,"ERROR: Rounded balance broken",IF(AI4&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C4&gt;0,W4=0),AND(E4&gt;0,Y4=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG4&gt;AH4,"ERROR: Rounded balance broken",IF(AND(J4&gt;0,AI4&lt;Settings!$B$2*J4/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -9422,7 +9422,7 @@
         <v/>
       </c>
       <c r="AJ5">
-        <f>IF(OR(AND(C5&gt;0,W5=0),AND(E5&gt;0,Y5=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG5&gt;AH5,"ERROR: Rounded balance broken",IF(AI5&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C5&gt;0,W5=0),AND(E5&gt;0,Y5=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG5&gt;AH5,"ERROR: Rounded balance broken",IF(AND(J5&gt;0,AI5&lt;Settings!$B$2*J5/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -9567,7 +9567,7 @@
         <v/>
       </c>
       <c r="AJ6">
-        <f>IF(OR(AND(C6&gt;0,W6=0),AND(E6&gt;0,Y6=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG6&gt;AH6,"ERROR: Rounded balance broken",IF(AI6&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C6&gt;0,W6=0),AND(E6&gt;0,Y6=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG6&gt;AH6,"ERROR: Rounded balance broken",IF(AND(J6&gt;0,AI6&lt;Settings!$B$2*J6/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -9712,7 +9712,7 @@
         <v/>
       </c>
       <c r="AJ7">
-        <f>IF(OR(AND(C7&gt;0,W7=0),AND(E7&gt;0,Y7=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG7&gt;AH7,"ERROR: Rounded balance broken",IF(AI7&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C7&gt;0,W7=0),AND(E7&gt;0,Y7=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG7&gt;AH7,"ERROR: Rounded balance broken",IF(AND(J7&gt;0,AI7&lt;Settings!$B$2*J7/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -9857,7 +9857,7 @@
         <v/>
       </c>
       <c r="AJ8">
-        <f>IF(OR(AND(C8&gt;0,W8=0),AND(E8&gt;0,Y8=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG8&gt;AH8,"ERROR: Rounded balance broken",IF(AI8&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C8&gt;0,W8=0),AND(E8&gt;0,Y8=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG8&gt;AH8,"ERROR: Rounded balance broken",IF(AND(J8&gt;0,AI8&lt;Settings!$B$2*J8/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -10002,7 +10002,7 @@
         <v/>
       </c>
       <c r="AJ9">
-        <f>IF(OR(AND(C9&gt;0,W9=0),AND(E9&gt;0,Y9=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG9&gt;AH9,"ERROR: Rounded balance broken",IF(AI9&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C9&gt;0,W9=0),AND(E9&gt;0,Y9=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG9&gt;AH9,"ERROR: Rounded balance broken",IF(AND(J9&gt;0,AI9&lt;Settings!$B$2*J9/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -10147,7 +10147,7 @@
         <v/>
       </c>
       <c r="AJ10">
-        <f>IF(OR(AND(C10&gt;0,W10=0),AND(E10&gt;0,Y10=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG10&gt;AH10,"ERROR: Rounded balance broken",IF(AI10&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C10&gt;0,W10=0),AND(E10&gt;0,Y10=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG10&gt;AH10,"ERROR: Rounded balance broken",IF(AND(J10&gt;0,AI10&lt;Settings!$B$2*J10/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -10292,7 +10292,7 @@
         <v/>
       </c>
       <c r="AJ11">
-        <f>IF(OR(AND(C11&gt;0,W11=0),AND(E11&gt;0,Y11=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG11&gt;AH11,"ERROR: Rounded balance broken",IF(AI11&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C11&gt;0,W11=0),AND(E11&gt;0,Y11=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG11&gt;AH11,"ERROR: Rounded balance broken",IF(AND(J11&gt;0,AI11&lt;Settings!$B$2*J11/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -10437,7 +10437,7 @@
         <v/>
       </c>
       <c r="AJ12">
-        <f>IF(OR(AND(C12&gt;0,W12=0),AND(E12&gt;0,Y12=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG12&gt;AH12,"ERROR: Rounded balance broken",IF(AI12&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C12&gt;0,W12=0),AND(E12&gt;0,Y12=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG12&gt;AH12,"ERROR: Rounded balance broken",IF(AND(J12&gt;0,AI12&lt;Settings!$B$2*J12/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -10582,7 +10582,7 @@
         <v/>
       </c>
       <c r="AJ13">
-        <f>IF(OR(AND(C13&gt;0,W13=0),AND(E13&gt;0,Y13=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG13&gt;AH13,"ERROR: Rounded balance broken",IF(AI13&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C13&gt;0,W13=0),AND(E13&gt;0,Y13=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG13&gt;AH13,"ERROR: Rounded balance broken",IF(AND(J13&gt;0,AI13&lt;Settings!$B$2*J13/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -10727,7 +10727,7 @@
         <v/>
       </c>
       <c r="AJ14">
-        <f>IF(OR(AND(C14&gt;0,W14=0),AND(E14&gt;0,Y14=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG14&gt;AH14,"ERROR: Rounded balance broken",IF(AI14&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C14&gt;0,W14=0),AND(E14&gt;0,Y14=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG14&gt;AH14,"ERROR: Rounded balance broken",IF(AND(J14&gt;0,AI14&lt;Settings!$B$2*J14/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -10872,7 +10872,7 @@
         <v/>
       </c>
       <c r="AJ15">
-        <f>IF(OR(AND(C15&gt;0,W15=0),AND(E15&gt;0,Y15=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG15&gt;AH15,"ERROR: Rounded balance broken",IF(AI15&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C15&gt;0,W15=0),AND(E15&gt;0,Y15=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG15&gt;AH15,"ERROR: Rounded balance broken",IF(AND(J15&gt;0,AI15&lt;Settings!$B$2*J15/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -11017,7 +11017,7 @@
         <v/>
       </c>
       <c r="AJ16">
-        <f>IF(OR(AND(C16&gt;0,W16=0),AND(E16&gt;0,Y16=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG16&gt;AH16,"ERROR: Rounded balance broken",IF(AI16&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C16&gt;0,W16=0),AND(E16&gt;0,Y16=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG16&gt;AH16,"ERROR: Rounded balance broken",IF(AND(J16&gt;0,AI16&lt;Settings!$B$2*J16/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -11162,7 +11162,7 @@
         <v/>
       </c>
       <c r="AJ17">
-        <f>IF(OR(AND(C17&gt;0,W17=0),AND(E17&gt;0,Y17=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG17&gt;AH17,"ERROR: Rounded balance broken",IF(AI17&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C17&gt;0,W17=0),AND(E17&gt;0,Y17=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG17&gt;AH17,"ERROR: Rounded balance broken",IF(AND(J17&gt;0,AI17&lt;Settings!$B$2*J17/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -11307,7 +11307,7 @@
         <v/>
       </c>
       <c r="AJ18">
-        <f>IF(OR(AND(C18&gt;0,W18=0),AND(E18&gt;0,Y18=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG18&gt;AH18,"ERROR: Rounded balance broken",IF(AI18&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C18&gt;0,W18=0),AND(E18&gt;0,Y18=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG18&gt;AH18,"ERROR: Rounded balance broken",IF(AND(J18&gt;0,AI18&lt;Settings!$B$2*J18/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -11452,7 +11452,7 @@
         <v/>
       </c>
       <c r="AJ19">
-        <f>IF(OR(AND(C19&gt;0,W19=0),AND(E19&gt;0,Y19=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG19&gt;AH19,"ERROR: Rounded balance broken",IF(AI19&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C19&gt;0,W19=0),AND(E19&gt;0,Y19=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG19&gt;AH19,"ERROR: Rounded balance broken",IF(AND(J19&gt;0,AI19&lt;Settings!$B$2*J19/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -11597,7 +11597,7 @@
         <v/>
       </c>
       <c r="AJ20">
-        <f>IF(OR(AND(C20&gt;0,W20=0),AND(E20&gt;0,Y20=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG20&gt;AH20,"ERROR: Rounded balance broken",IF(AI20&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C20&gt;0,W20=0),AND(E20&gt;0,Y20=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG20&gt;AH20,"ERROR: Rounded balance broken",IF(AND(J20&gt;0,AI20&lt;Settings!$B$2*J20/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -11742,7 +11742,7 @@
         <v/>
       </c>
       <c r="AJ21">
-        <f>IF(OR(AND(C21&gt;0,W21=0),AND(E21&gt;0,Y21=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG21&gt;AH21,"ERROR: Rounded balance broken",IF(AI21&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C21&gt;0,W21=0),AND(E21&gt;0,Y21=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG21&gt;AH21,"ERROR: Rounded balance broken",IF(AND(J21&gt;0,AI21&lt;Settings!$B$2*J21/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -11887,7 +11887,7 @@
         <v/>
       </c>
       <c r="AJ22">
-        <f>IF(OR(AND(C22&gt;0,W22=0),AND(E22&gt;0,Y22=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG22&gt;AH22,"ERROR: Rounded balance broken",IF(AI22&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C22&gt;0,W22=0),AND(E22&gt;0,Y22=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG22&gt;AH22,"ERROR: Rounded balance broken",IF(AND(J22&gt;0,AI22&lt;Settings!$B$2*J22/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -12032,7 +12032,7 @@
         <v/>
       </c>
       <c r="AJ23">
-        <f>IF(OR(AND(C23&gt;0,W23=0),AND(E23&gt;0,Y23=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG23&gt;AH23,"ERROR: Rounded balance broken",IF(AI23&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C23&gt;0,W23=0),AND(E23&gt;0,Y23=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG23&gt;AH23,"ERROR: Rounded balance broken",IF(AND(J23&gt;0,AI23&lt;Settings!$B$2*J23/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -12177,7 +12177,7 @@
         <v/>
       </c>
       <c r="AJ24">
-        <f>IF(OR(AND(C24&gt;0,W24=0),AND(E24&gt;0,Y24=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG24&gt;AH24,"ERROR: Rounded balance broken",IF(AI24&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C24&gt;0,W24=0),AND(E24&gt;0,Y24=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG24&gt;AH24,"ERROR: Rounded balance broken",IF(AND(J24&gt;0,AI24&lt;Settings!$B$2*J24/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -12322,7 +12322,7 @@
         <v/>
       </c>
       <c r="AJ25">
-        <f>IF(OR(AND(C25&gt;0,W25=0),AND(E25&gt;0,Y25=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG25&gt;AH25,"ERROR: Rounded balance broken",IF(AI25&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C25&gt;0,W25=0),AND(E25&gt;0,Y25=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG25&gt;AH25,"ERROR: Rounded balance broken",IF(AND(J25&gt;0,AI25&lt;Settings!$B$2*J25/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -12467,7 +12467,7 @@
         <v/>
       </c>
       <c r="AJ26">
-        <f>IF(OR(AND(C26&gt;0,W26=0),AND(E26&gt;0,Y26=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG26&gt;AH26,"ERROR: Rounded balance broken",IF(AI26&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C26&gt;0,W26=0),AND(E26&gt;0,Y26=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG26&gt;AH26,"ERROR: Rounded balance broken",IF(AND(J26&gt;0,AI26&lt;Settings!$B$2*J26/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -12612,7 +12612,7 @@
         <v/>
       </c>
       <c r="AJ27">
-        <f>IF(OR(AND(C27&gt;0,W27=0),AND(E27&gt;0,Y27=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG27&gt;AH27,"ERROR: Rounded balance broken",IF(AI27&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C27&gt;0,W27=0),AND(E27&gt;0,Y27=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG27&gt;AH27,"ERROR: Rounded balance broken",IF(AND(J27&gt;0,AI27&lt;Settings!$B$2*J27/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -12757,7 +12757,7 @@
         <v/>
       </c>
       <c r="AJ28">
-        <f>IF(OR(AND(C28&gt;0,W28=0),AND(E28&gt;0,Y28=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG28&gt;AH28,"ERROR: Rounded balance broken",IF(AI28&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C28&gt;0,W28=0),AND(E28&gt;0,Y28=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG28&gt;AH28,"ERROR: Rounded balance broken",IF(AND(J28&gt;0,AI28&lt;Settings!$B$2*J28/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -12902,7 +12902,7 @@
         <v/>
       </c>
       <c r="AJ29">
-        <f>IF(OR(AND(C29&gt;0,W29=0),AND(E29&gt;0,Y29=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG29&gt;AH29,"ERROR: Rounded balance broken",IF(AI29&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C29&gt;0,W29=0),AND(E29&gt;0,Y29=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG29&gt;AH29,"ERROR: Rounded balance broken",IF(AND(J29&gt;0,AI29&lt;Settings!$B$2*J29/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -13047,7 +13047,7 @@
         <v/>
       </c>
       <c r="AJ30">
-        <f>IF(OR(AND(C30&gt;0,W30=0),AND(E30&gt;0,Y30=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG30&gt;AH30,"ERROR: Rounded balance broken",IF(AI30&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C30&gt;0,W30=0),AND(E30&gt;0,Y30=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG30&gt;AH30,"ERROR: Rounded balance broken",IF(AND(J30&gt;0,AI30&lt;Settings!$B$2*J30/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -13192,7 +13192,7 @@
         <v/>
       </c>
       <c r="AJ31">
-        <f>IF(OR(AND(C31&gt;0,W31=0),AND(E31&gt;0,Y31=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG31&gt;AH31,"ERROR: Rounded balance broken",IF(AI31&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C31&gt;0,W31=0),AND(E31&gt;0,Y31=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG31&gt;AH31,"ERROR: Rounded balance broken",IF(AND(J31&gt;0,AI31&lt;Settings!$B$2*J31/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -13337,7 +13337,7 @@
         <v/>
       </c>
       <c r="AJ32">
-        <f>IF(OR(AND(C32&gt;0,W32=0),AND(E32&gt;0,Y32=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG32&gt;AH32,"ERROR: Rounded balance broken",IF(AI32&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C32&gt;0,W32=0),AND(E32&gt;0,Y32=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG32&gt;AH32,"ERROR: Rounded balance broken",IF(AND(J32&gt;0,AI32&lt;Settings!$B$2*J32/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -13482,7 +13482,7 @@
         <v/>
       </c>
       <c r="AJ33">
-        <f>IF(OR(AND(C33&gt;0,W33=0),AND(E33&gt;0,Y33=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG33&gt;AH33,"ERROR: Rounded balance broken",IF(AI33&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C33&gt;0,W33=0),AND(E33&gt;0,Y33=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG33&gt;AH33,"ERROR: Rounded balance broken",IF(AND(J33&gt;0,AI33&lt;Settings!$B$2*J33/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -13627,7 +13627,7 @@
         <v/>
       </c>
       <c r="AJ34">
-        <f>IF(OR(AND(C34&gt;0,W34=0),AND(E34&gt;0,Y34=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG34&gt;AH34,"ERROR: Rounded balance broken",IF(AI34&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C34&gt;0,W34=0),AND(E34&gt;0,Y34=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG34&gt;AH34,"ERROR: Rounded balance broken",IF(AND(J34&gt;0,AI34&lt;Settings!$B$2*J34/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -13772,7 +13772,7 @@
         <v/>
       </c>
       <c r="AJ35">
-        <f>IF(OR(AND(C35&gt;0,W35=0),AND(E35&gt;0,Y35=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG35&gt;AH35,"ERROR: Rounded balance broken",IF(AI35&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C35&gt;0,W35=0),AND(E35&gt;0,Y35=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG35&gt;AH35,"ERROR: Rounded balance broken",IF(AND(J35&gt;0,AI35&lt;Settings!$B$2*J35/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -13917,7 +13917,7 @@
         <v/>
       </c>
       <c r="AJ36">
-        <f>IF(OR(AND(C36&gt;0,W36=0),AND(E36&gt;0,Y36=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG36&gt;AH36,"ERROR: Rounded balance broken",IF(AI36&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C36&gt;0,W36=0),AND(E36&gt;0,Y36=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG36&gt;AH36,"ERROR: Rounded balance broken",IF(AND(J36&gt;0,AI36&lt;Settings!$B$2*J36/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -14062,7 +14062,7 @@
         <v/>
       </c>
       <c r="AJ37">
-        <f>IF(OR(AND(C37&gt;0,W37=0),AND(E37&gt;0,Y37=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG37&gt;AH37,"ERROR: Rounded balance broken",IF(AI37&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C37&gt;0,W37=0),AND(E37&gt;0,Y37=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG37&gt;AH37,"ERROR: Rounded balance broken",IF(AND(J37&gt;0,AI37&lt;Settings!$B$2*J37/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -14207,7 +14207,7 @@
         <v/>
       </c>
       <c r="AJ38">
-        <f>IF(OR(AND(C38&gt;0,W38=0),AND(E38&gt;0,Y38=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG38&gt;AH38,"ERROR: Rounded balance broken",IF(AI38&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C38&gt;0,W38=0),AND(E38&gt;0,Y38=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG38&gt;AH38,"ERROR: Rounded balance broken",IF(AND(J38&gt;0,AI38&lt;Settings!$B$2*J38/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -14352,7 +14352,7 @@
         <v/>
       </c>
       <c r="AJ39">
-        <f>IF(OR(AND(C39&gt;0,W39=0),AND(E39&gt;0,Y39=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG39&gt;AH39,"ERROR: Rounded balance broken",IF(AI39&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C39&gt;0,W39=0),AND(E39&gt;0,Y39=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG39&gt;AH39,"ERROR: Rounded balance broken",IF(AND(J39&gt;0,AI39&lt;Settings!$B$2*J39/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -14497,7 +14497,7 @@
         <v/>
       </c>
       <c r="AJ40">
-        <f>IF(OR(AND(C40&gt;0,W40=0),AND(E40&gt;0,Y40=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG40&gt;AH40,"ERROR: Rounded balance broken",IF(AI40&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C40&gt;0,W40=0),AND(E40&gt;0,Y40=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG40&gt;AH40,"ERROR: Rounded balance broken",IF(AND(J40&gt;0,AI40&lt;Settings!$B$2*J40/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -14642,7 +14642,7 @@
         <v/>
       </c>
       <c r="AJ41">
-        <f>IF(OR(AND(C41&gt;0,W41=0),AND(E41&gt;0,Y41=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG41&gt;AH41,"ERROR: Rounded balance broken",IF(AI41&lt;Settings!$B$2*Settings!$B$7/100,"WARNING","OK")))</f>
+        <f>IF(OR(AND(C41&gt;0,W41=0),AND(E41&gt;0,Y41=0),Settings!$B$2&lt;Settings!$B$5),"ERROR: LotStep too coarse",IF(AG41&gt;AH41,"ERROR: Rounded balance broken",IF(AND(J41&gt;0,AI41&lt;Settings!$B$2*J41/100),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -14710,7 +14710,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>INDEX(DownTrend!Q:Q,Settings!B4+3)</f>
+        <f>IF(Settings!$B$10="DOWN",INDEX(DownTrend!Q:Q,Settings!B4+3),INDEX(UpTrend!R:R,Settings!B4+3))</f>
         <v/>
       </c>
     </row>
@@ -14721,7 +14721,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>INDEX(DownTrend!R:R,Settings!B4+3)</f>
+        <f>IF(Settings!$B$10="DOWN",INDEX(DownTrend!R:R,Settings!B4+3),INDEX(UpTrend!Q:Q,Settings!B4+3))</f>
         <v/>
       </c>
     </row>
@@ -14732,7 +14732,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>INDEX(DownTrend!S:S,Settings!B4+3)</f>
+        <f>IF(Settings!$B$10="DOWN",INDEX(DownTrend!S:S,Settings!B4+3),INDEX(UpTrend!S:S,Settings!B4+3))</f>
         <v/>
       </c>
     </row>
@@ -14743,7 +14743,7 @@
         </is>
       </c>
       <c r="B8">
-        <f>INDEX(DownTrend!N:N,Settings!B4+3)</f>
+        <f>IF(Settings!$B$10="DOWN",INDEX(DownTrend!N:N,Settings!B4+3),INDEX(UpTrend!N:N,Settings!B4+3))</f>
         <v/>
       </c>
     </row>
@@ -14820,7 +14820,7 @@
         </is>
       </c>
       <c r="B15">
-        <f>IF(COUNTIF(DownTrend!T3:INDEX(DownTrend!T:T,Settings!B4+3),"ERROR*")+COUNTIF(UpTrend!T3:INDEX(UpTrend!T:T,Settings!B4+3),"ERROR*")&gt;0,"ERROR",IF(COUNTIF(DownTrend!T3:INDEX(DownTrend!T:T,Settings!B4+3),"WARNING*")+COUNTIF(UpTrend!T3:INDEX(UpTrend!T:T,Settings!B4+3),"WARNING*")&gt;0,"WARNING","OK"))</f>
+        <f>IF(Settings!$B$10="DOWN",IF(OR(INDEX(DownTrend!T:T,Settings!B4+3)="ERROR: Rounding broke protection balance",LEFT(INDEX(DownTrend!AJ:AJ,Settings!B4+3),5)="ERROR"),"ERROR",IF(OR(LEFT(INDEX(DownTrend!T:T,Settings!B4+3),7)="WARNING",INDEX(DownTrend!AJ:AJ,Settings!B4+3)="WARNING"),"WARNING","OK")),IF(OR(INDEX(UpTrend!T:T,Settings!B4+3)="ERROR: Rounding broke protection balance",LEFT(INDEX(UpTrend!AJ:AJ,Settings!B4+3),5)="ERROR"),"ERROR",IF(OR(LEFT(INDEX(UpTrend!T:T,Settings!B4+3),7)="WARNING",INDEX(UpTrend!AJ:AJ,Settings!B4+3)="WARNING"),"WARNING","OK")))</f>
         <v/>
       </c>
     </row>
@@ -14831,7 +14831,7 @@
         </is>
       </c>
       <c r="B16">
-        <f>IF(COUNTIF(DownTrend!AJ3:INDEX(DownTrend!AJ:AJ,Settings!B4+3),"ERROR*")+COUNTIF(UpTrend!AJ3:INDEX(UpTrend!AJ:AJ,Settings!B4+3),"ERROR*")&gt;0,"ERROR",IF(COUNTIF(DownTrend!AJ3:INDEX(DownTrend!AJ:AJ,Settings!B4+3),"WARNING*")+COUNTIF(UpTrend!AJ3:INDEX(UpTrend!AJ:AJ,Settings!B4+3),"WARNING*")&gt;0,"WARNING","OK"))</f>
+        <f>IF(Settings!$B$10="DOWN",INDEX(DownTrend!AJ:AJ,Settings!B4+3),INDEX(UpTrend!AJ:AJ,Settings!B4+3))</f>
         <v/>
       </c>
     </row>

</xml_diff>